<commit_message>
Automatisches Update TM + Transfers - 11.06.2025 08:25
</commit_message>
<xml_diff>
--- a/TM_all.xlsx
+++ b/TM_all.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/aecf56309e6168f4/Documents/comunio/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="214" documentId="8_{B00F7E9F-5C85-449B-834E-0179FBCEE2D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{45D9059B-905C-4C1F-88CF-0CDFBF289F64}"/>
+  <xr:revisionPtr revIDLastSave="218" documentId="8_{B00F7E9F-5C85-449B-834E-0179FBCEE2D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{87486627-A459-446D-A33B-5F6E3A2DD1D1}"/>
   <bookViews>
     <workbookView xWindow="2110" yWindow="2130" windowWidth="28800" windowHeight="15370" xr2:uid="{607DE709-F91E-4262-9941-1066BBEC319E}"/>
   </bookViews>
@@ -860,7 +860,7 @@
     <t>Diks</t>
   </si>
   <si>
-    <t>11.06.2026</t>
+    <t>11.06.2025</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Automatisches Update TM + Transfers - 13.06.2025 21:20
</commit_message>
<xml_diff>
--- a/TM_all.xlsx
+++ b/TM_all.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/aecf56309e6168f4/Documents/comunio/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="225" documentId="8_{B00F7E9F-5C85-449B-834E-0179FBCEE2D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6B04FA23-EC55-4F77-88BC-456F87E4EAD1}"/>
+  <xr:revisionPtr revIDLastSave="234" documentId="8_{B00F7E9F-5C85-449B-834E-0179FBCEE2D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{51C20D1E-0DF0-489C-83F1-A6D45CB1609D}"/>
   <bookViews>
-    <workbookView xWindow="2110" yWindow="2130" windowWidth="28800" windowHeight="15370" xr2:uid="{607DE709-F91E-4262-9941-1066BBEC319E}"/>
+    <workbookView xWindow="6660" yWindow="2700" windowWidth="28800" windowHeight="15370" xr2:uid="{607DE709-F91E-4262-9941-1066BBEC319E}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7275" uniqueCount="281">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7987" uniqueCount="295">
   <si>
     <t>Spieler</t>
   </si>
@@ -883,6 +883,48 @@
   <si>
     <t>12.06.2025</t>
   </si>
+  <si>
+    <t>W. Orbán</t>
+  </si>
+  <si>
+    <t>5,7</t>
+  </si>
+  <si>
+    <t>Kramarić</t>
+  </si>
+  <si>
+    <t>Kainz</t>
+  </si>
+  <si>
+    <t>3,7</t>
+  </si>
+  <si>
+    <t>Burkardt</t>
+  </si>
+  <si>
+    <t>6,6</t>
+  </si>
+  <si>
+    <t>Jäkel</t>
+  </si>
+  <si>
+    <t>Caci</t>
+  </si>
+  <si>
+    <t>Dietz</t>
+  </si>
+  <si>
+    <t>0,7</t>
+  </si>
+  <si>
+    <t>Malatini</t>
+  </si>
+  <si>
+    <t>Sieb</t>
+  </si>
+  <si>
+    <t>13.06.2025</t>
+  </si>
 </sst>
 </file>
 
@@ -1306,7 +1348,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{93EB6F54-7766-4759-97DF-03549A275A7C}">
-  <dimension ref="A1:M1045"/>
+  <dimension ref="A1:M1135"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.90625" style="2"/>
@@ -40345,7 +40387,7 @@
         <v>280</v>
       </c>
     </row>
-    <row r="1041" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="1041" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B1041" s="2" t="s">
         <v>206</v>
       </c>
@@ -40383,7 +40425,7 @@
         <v>280</v>
       </c>
     </row>
-    <row r="1042" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="1042" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B1042" s="2" t="s">
         <v>118</v>
       </c>
@@ -40421,7 +40463,7 @@
         <v>280</v>
       </c>
     </row>
-    <row r="1043" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="1043" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B1043" s="2" t="s">
         <v>121</v>
       </c>
@@ -40459,7 +40501,7 @@
         <v>280</v>
       </c>
     </row>
-    <row r="1044" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="1044" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B1044" s="2" t="s">
         <v>200</v>
       </c>
@@ -40497,7 +40539,7 @@
         <v>280</v>
       </c>
     </row>
-    <row r="1045" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="1045" spans="1:13" ht="13" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B1045" s="2" t="s">
         <v>272</v>
       </c>
@@ -40534,6 +40576,3480 @@
       <c r="M1045" s="7" t="s">
         <v>280</v>
       </c>
+    </row>
+    <row r="1046" spans="1:13" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1046" s="6"/>
+      <c r="B1046" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1046" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1046" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1046" s="2">
+        <v>70</v>
+      </c>
+      <c r="F1046" s="2">
+        <v>1890000</v>
+      </c>
+      <c r="G1046" s="2">
+        <v>1890000</v>
+      </c>
+      <c r="H1046" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="I1046" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1046" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1046" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1046" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="M1046" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1047" spans="1:13" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1047" s="6"/>
+      <c r="B1047" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="C1047" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1047" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="E1047" s="2">
+        <v>124</v>
+      </c>
+      <c r="F1047" s="2">
+        <v>5870000</v>
+      </c>
+      <c r="G1047" s="2">
+        <v>5640000</v>
+      </c>
+      <c r="H1047" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="I1047" s="2" t="s">
+        <v>274</v>
+      </c>
+      <c r="J1047" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1047" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1047" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="M1047" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1048" spans="1:13" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1048" s="6"/>
+      <c r="B1048" s="2" t="s">
+        <v>281</v>
+      </c>
+      <c r="C1048" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1048" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="E1048" s="2">
+        <v>143</v>
+      </c>
+      <c r="F1048" s="2">
+        <v>6270000</v>
+      </c>
+      <c r="G1048" s="2">
+        <v>6170000</v>
+      </c>
+      <c r="H1048" s="2" t="s">
+        <v>282</v>
+      </c>
+      <c r="I1048" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1048" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1048" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1048" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="M1048" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1049" spans="1:13" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1049" s="6"/>
+      <c r="B1049" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="C1049" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1049" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E1049" s="2">
+        <v>128</v>
+      </c>
+      <c r="F1049" s="2">
+        <v>4790000</v>
+      </c>
+      <c r="G1049" s="2">
+        <v>4680000</v>
+      </c>
+      <c r="H1049" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="I1049" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1049" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1049" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1049" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="M1049" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1050" spans="1:13" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1050" s="6"/>
+      <c r="B1050" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="C1050" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1050" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="E1050" s="2">
+        <v>83</v>
+      </c>
+      <c r="F1050" s="2">
+        <v>1040000</v>
+      </c>
+      <c r="G1050" s="2">
+        <v>1050000</v>
+      </c>
+      <c r="H1050" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="I1050" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1050" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1050" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1050" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="M1050" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1051" spans="1:13" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1051" s="6"/>
+      <c r="B1051" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1051" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1051" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E1051" s="2">
+        <v>43</v>
+      </c>
+      <c r="F1051" s="2">
+        <v>2460000</v>
+      </c>
+      <c r="G1051" s="2">
+        <v>2460000</v>
+      </c>
+      <c r="H1051" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="I1051" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1051" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1051" s="2">
+        <v>1</v>
+      </c>
+      <c r="L1051" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="M1051" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1052" spans="1:13" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1052" s="6"/>
+      <c r="B1052" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1052" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1052" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E1052" s="2">
+        <v>42</v>
+      </c>
+      <c r="F1052" s="2">
+        <v>5020000</v>
+      </c>
+      <c r="G1052" s="2">
+        <v>4970000</v>
+      </c>
+      <c r="H1052" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="I1052" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1052" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1052" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1052" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="M1052" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1053" spans="1:13" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1053" s="6"/>
+      <c r="B1053" s="2" t="s">
+        <v>220</v>
+      </c>
+      <c r="C1053" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1053" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="E1053" s="2">
+        <v>43</v>
+      </c>
+      <c r="F1053" s="2">
+        <v>4330000</v>
+      </c>
+      <c r="G1053" s="2">
+        <v>4350000</v>
+      </c>
+      <c r="H1053" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="I1053" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1053" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="K1053" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1053" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="M1053" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1054" spans="1:13" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1054" s="6"/>
+      <c r="B1054" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="C1054" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1054" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="E1054" s="2">
+        <v>60</v>
+      </c>
+      <c r="F1054" s="2">
+        <v>1360000</v>
+      </c>
+      <c r="G1054" s="2">
+        <v>1350000</v>
+      </c>
+      <c r="H1054" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="I1054" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1054" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1054" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1054" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="M1054" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1055" spans="1:13" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1055" s="6"/>
+      <c r="B1055" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C1055" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1055" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="E1055" s="2">
+        <v>124</v>
+      </c>
+      <c r="F1055" s="2">
+        <v>3370000</v>
+      </c>
+      <c r="G1055" s="2">
+        <v>3260000</v>
+      </c>
+      <c r="H1055" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="I1055" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1055" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1055" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1055" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="M1055" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1056" spans="1:13" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1056" s="6"/>
+      <c r="B1056" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1056" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1056" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E1056" s="2">
+        <v>112</v>
+      </c>
+      <c r="F1056" s="2">
+        <v>4560000</v>
+      </c>
+      <c r="G1056" s="2">
+        <v>4530000</v>
+      </c>
+      <c r="H1056" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="I1056" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1056" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1056" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1056" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="M1056" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1057" spans="1:13" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1057" s="6"/>
+      <c r="B1057" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="C1057" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1057" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="E1057" s="2">
+        <v>108</v>
+      </c>
+      <c r="F1057" s="2">
+        <v>3620000</v>
+      </c>
+      <c r="G1057" s="2">
+        <v>3560000</v>
+      </c>
+      <c r="H1057" s="2" t="s">
+        <v>264</v>
+      </c>
+      <c r="I1057" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1057" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1057" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1057" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="M1057" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1058" spans="1:13" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1058" s="6"/>
+      <c r="B1058" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="C1058" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1058" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="E1058" s="2">
+        <v>183</v>
+      </c>
+      <c r="F1058" s="2">
+        <v>10130000</v>
+      </c>
+      <c r="G1058" s="2">
+        <v>10020000</v>
+      </c>
+      <c r="H1058" s="2" t="s">
+        <v>236</v>
+      </c>
+      <c r="I1058" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1058" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="K1058" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1058" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="M1058" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1059" spans="1:13" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1059" s="6"/>
+      <c r="B1059" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="C1059" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1059" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E1059" s="2">
+        <v>167</v>
+      </c>
+      <c r="F1059" s="2">
+        <v>9680000</v>
+      </c>
+      <c r="G1059" s="2">
+        <v>9530000</v>
+      </c>
+      <c r="H1059" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="I1059" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1059" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1059" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1059" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="M1059" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1060" spans="1:13" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1060" s="6"/>
+      <c r="B1060" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C1060" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1060" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="E1060" s="2">
+        <v>127</v>
+      </c>
+      <c r="F1060" s="2">
+        <v>3230000</v>
+      </c>
+      <c r="G1060" s="2">
+        <v>3210000</v>
+      </c>
+      <c r="H1060" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="I1060" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1060" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1060" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1060" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="M1060" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1061" spans="1:13" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1061" s="6"/>
+      <c r="B1061" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="C1061" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1061" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E1061" s="2">
+        <v>69</v>
+      </c>
+      <c r="F1061" s="2">
+        <v>1730000</v>
+      </c>
+      <c r="G1061" s="2">
+        <v>1740000</v>
+      </c>
+      <c r="H1061" s="2" t="s">
+        <v>241</v>
+      </c>
+      <c r="I1061" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1061" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1061" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1061" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="M1061" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1062" spans="1:13" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1062" s="6"/>
+      <c r="B1062" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C1062" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1062" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="E1062" s="2">
+        <v>72</v>
+      </c>
+      <c r="F1062" s="2">
+        <v>1840000</v>
+      </c>
+      <c r="G1062" s="2">
+        <v>1840000</v>
+      </c>
+      <c r="H1062" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="I1062" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1062" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1062" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1062" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="M1062" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1063" spans="1:13" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1063" s="6"/>
+      <c r="B1063" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="C1063" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1063" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="E1063" s="2">
+        <v>0</v>
+      </c>
+      <c r="F1063" s="2">
+        <v>2430000</v>
+      </c>
+      <c r="G1063" s="2">
+        <v>2410000</v>
+      </c>
+      <c r="H1063" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="I1063" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1063" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1063" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1063" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="M1063" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1064" spans="1:13" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1064" s="6"/>
+      <c r="B1064" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="C1064" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1064" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="E1064" s="2">
+        <v>0</v>
+      </c>
+      <c r="F1064" s="2">
+        <v>2340000</v>
+      </c>
+      <c r="G1064" s="2">
+        <v>2340000</v>
+      </c>
+      <c r="H1064" s="2" t="s">
+        <v>244</v>
+      </c>
+      <c r="I1064" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1064" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="K1064" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1064" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="M1064" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1065" spans="1:13" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1065" s="6"/>
+      <c r="B1065" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C1065" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1065" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="E1065" s="2">
+        <v>110</v>
+      </c>
+      <c r="F1065" s="2">
+        <v>3490000</v>
+      </c>
+      <c r="G1065" s="2">
+        <v>3410000</v>
+      </c>
+      <c r="H1065" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="I1065" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1065" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1065" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1065" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="M1065" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1066" spans="1:13" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1066" s="6"/>
+      <c r="B1066" s="2" t="s">
+        <v>284</v>
+      </c>
+      <c r="C1066" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1066" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1066" s="2">
+        <v>0</v>
+      </c>
+      <c r="F1066" s="2">
+        <v>3740000</v>
+      </c>
+      <c r="G1066" s="2">
+        <v>3750000</v>
+      </c>
+      <c r="H1066" s="2" t="s">
+        <v>285</v>
+      </c>
+      <c r="I1066" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1066" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1066" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1066" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="M1066" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1067" spans="1:13" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1067" s="6"/>
+      <c r="B1067" s="2" t="s">
+        <v>275</v>
+      </c>
+      <c r="C1067" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1067" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="E1067" s="2">
+        <v>59</v>
+      </c>
+      <c r="F1067" s="2">
+        <v>900000</v>
+      </c>
+      <c r="G1067" s="2">
+        <v>910000</v>
+      </c>
+      <c r="H1067" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="I1067" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1067" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1067" s="2">
+        <v>1</v>
+      </c>
+      <c r="L1067" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1067" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1068" spans="1:13" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1068" s="6"/>
+      <c r="B1068" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C1068" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1068" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1068" s="2">
+        <v>0</v>
+      </c>
+      <c r="F1068" s="2">
+        <v>3160000</v>
+      </c>
+      <c r="G1068" s="2">
+        <v>3080000</v>
+      </c>
+      <c r="H1068" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="I1068" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1068" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1068" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1068" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="M1068" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1069" spans="1:13" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1069" s="6"/>
+      <c r="B1069" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="C1069" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1069" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="E1069" s="2">
+        <v>95</v>
+      </c>
+      <c r="F1069" s="2">
+        <v>3670000</v>
+      </c>
+      <c r="G1069" s="2">
+        <v>3630000</v>
+      </c>
+      <c r="H1069" s="2" t="s">
+        <v>285</v>
+      </c>
+      <c r="I1069" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1069" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1069" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1069" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="M1069" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1070" spans="1:13" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1070" s="6"/>
+      <c r="B1070" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="C1070" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1070" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="E1070" s="2">
+        <v>71</v>
+      </c>
+      <c r="F1070" s="2">
+        <v>1570000</v>
+      </c>
+      <c r="G1070" s="2">
+        <v>1600000</v>
+      </c>
+      <c r="H1070" s="2" t="s">
+        <v>238</v>
+      </c>
+      <c r="I1070" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1070" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1070" s="2">
+        <v>1</v>
+      </c>
+      <c r="L1070" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="M1070" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1071" spans="1:13" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1071" s="6"/>
+      <c r="B1071" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C1071" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1071" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="E1071" s="2">
+        <v>127</v>
+      </c>
+      <c r="F1071" s="2">
+        <v>5700000</v>
+      </c>
+      <c r="G1071" s="2">
+        <v>5620000</v>
+      </c>
+      <c r="H1071" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="I1071" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1071" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1071" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1071" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="M1071" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1072" spans="1:13" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1072" s="6"/>
+      <c r="B1072" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C1072" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1072" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="E1072" s="2">
+        <v>8</v>
+      </c>
+      <c r="F1072" s="2">
+        <v>230000</v>
+      </c>
+      <c r="G1072" s="2">
+        <v>230000</v>
+      </c>
+      <c r="H1072" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="I1072" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1072" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1072" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1072" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="M1072" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1073" spans="1:13" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1073" s="6"/>
+      <c r="B1073" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C1073" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1073" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="E1073" s="2">
+        <v>72</v>
+      </c>
+      <c r="F1073" s="2">
+        <v>3330000</v>
+      </c>
+      <c r="G1073" s="2">
+        <v>3260000</v>
+      </c>
+      <c r="H1073" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="I1073" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1073" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1073" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1073" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="M1073" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1074" spans="1:13" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1074" s="6"/>
+      <c r="B1074" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="C1074" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1074" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="E1074" s="2">
+        <v>36</v>
+      </c>
+      <c r="F1074" s="2">
+        <v>3150000</v>
+      </c>
+      <c r="G1074" s="2">
+        <v>3160000</v>
+      </c>
+      <c r="H1074" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="I1074" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1074" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="K1074" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1074" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="M1074" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1075" spans="1:13" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1075" s="6"/>
+      <c r="B1075" s="2" t="s">
+        <v>286</v>
+      </c>
+      <c r="C1075" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1075" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="E1075" s="2">
+        <v>184</v>
+      </c>
+      <c r="F1075" s="2">
+        <v>15530000</v>
+      </c>
+      <c r="G1075" s="2">
+        <v>15550000</v>
+      </c>
+      <c r="H1075" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="I1075" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1075" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1075" s="2">
+        <v>2</v>
+      </c>
+      <c r="L1075" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1075" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1076" spans="1:13" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1076" s="6"/>
+      <c r="B1076" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="C1076" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1076" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="E1076" s="2">
+        <v>87</v>
+      </c>
+      <c r="F1076" s="2">
+        <v>2590000</v>
+      </c>
+      <c r="G1076" s="2">
+        <v>2570000</v>
+      </c>
+      <c r="H1076" s="2" t="s">
+        <v>238</v>
+      </c>
+      <c r="I1076" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1076" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1076" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1076" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="M1076" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1077" spans="1:13" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1077" s="6"/>
+      <c r="B1077" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="C1077" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1077" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="E1077" s="2">
+        <v>123</v>
+      </c>
+      <c r="F1077" s="2">
+        <v>3760000</v>
+      </c>
+      <c r="G1077" s="2">
+        <v>3840000</v>
+      </c>
+      <c r="H1077" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="I1077" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1077" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1077" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1077" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="M1077" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1078" spans="1:13" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1078" s="6"/>
+      <c r="B1078" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="C1078" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1078" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="E1078" s="2">
+        <v>89</v>
+      </c>
+      <c r="F1078" s="2">
+        <v>1850000</v>
+      </c>
+      <c r="G1078" s="2">
+        <v>1860000</v>
+      </c>
+      <c r="H1078" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="I1078" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1078" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1078" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1078" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="M1078" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1079" spans="1:13" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1079" s="6"/>
+      <c r="B1079" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="C1079" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1079" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1079" s="2">
+        <v>0</v>
+      </c>
+      <c r="F1079" s="2">
+        <v>290000</v>
+      </c>
+      <c r="G1079" s="2">
+        <v>290000</v>
+      </c>
+      <c r="H1079" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="I1079" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1079" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="K1079" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1079" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1079" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1080" spans="1:13" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1080" s="6"/>
+      <c r="B1080" s="2" t="s">
+        <v>288</v>
+      </c>
+      <c r="C1080" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1080" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="E1080" s="2">
+        <v>0</v>
+      </c>
+      <c r="F1080" s="2">
+        <v>220000</v>
+      </c>
+      <c r="G1080" s="2">
+        <v>220000</v>
+      </c>
+      <c r="H1080" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="I1080" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1080" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="K1080" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1080" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1080" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1081" spans="1:13" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1081" s="6"/>
+      <c r="B1081" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="C1081" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1081" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="E1081" s="2">
+        <v>6</v>
+      </c>
+      <c r="F1081" s="2">
+        <v>3650000</v>
+      </c>
+      <c r="G1081" s="2">
+        <v>3720000</v>
+      </c>
+      <c r="H1081" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="I1081" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1081" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="K1081" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1081" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="M1081" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1082" spans="1:13" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1082" s="6"/>
+      <c r="B1082" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="C1082" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1082" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E1082" s="2">
+        <v>77</v>
+      </c>
+      <c r="F1082" s="2">
+        <v>2320000</v>
+      </c>
+      <c r="G1082" s="2">
+        <v>2270000</v>
+      </c>
+      <c r="H1082" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="I1082" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1082" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1082" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1082" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="M1082" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1083" spans="1:13" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1083" s="6"/>
+      <c r="B1083" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="C1083" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1083" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E1083" s="2">
+        <v>100</v>
+      </c>
+      <c r="F1083" s="2">
+        <v>4810000</v>
+      </c>
+      <c r="G1083" s="2">
+        <v>4870000</v>
+      </c>
+      <c r="H1083" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="I1083" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1083" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1083" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1083" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="M1083" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1084" spans="1:13" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1084" s="6"/>
+      <c r="B1084" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="C1084" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1084" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1084" s="2">
+        <v>199</v>
+      </c>
+      <c r="F1084" s="2">
+        <v>19070000</v>
+      </c>
+      <c r="G1084" s="2">
+        <v>19290000</v>
+      </c>
+      <c r="H1084" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="I1084" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1084" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1084" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1084" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="M1084" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1085" spans="1:13" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1085" s="6"/>
+      <c r="B1085" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="C1085" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1085" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="E1085" s="2">
+        <v>179</v>
+      </c>
+      <c r="F1085" s="2">
+        <v>11850000</v>
+      </c>
+      <c r="G1085" s="2">
+        <v>11790000</v>
+      </c>
+      <c r="H1085" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="I1085" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1085" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1085" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1085" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="M1085" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1086" spans="1:13" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1086" s="6"/>
+      <c r="B1086" s="2" t="s">
+        <v>276</v>
+      </c>
+      <c r="C1086" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1086" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E1086" s="2">
+        <v>7</v>
+      </c>
+      <c r="F1086" s="2">
+        <v>350000</v>
+      </c>
+      <c r="G1086" s="2">
+        <v>350000</v>
+      </c>
+      <c r="H1086" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="I1086" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1086" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1086" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1086" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1086" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1087" spans="1:13" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1087" s="6"/>
+      <c r="B1087" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="C1087" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1087" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E1087" s="2">
+        <v>185</v>
+      </c>
+      <c r="F1087" s="2">
+        <v>12210000</v>
+      </c>
+      <c r="G1087" s="2">
+        <v>12130000</v>
+      </c>
+      <c r="H1087" s="2" t="s">
+        <v>255</v>
+      </c>
+      <c r="I1087" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1087" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1087" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1087" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="M1087" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1088" spans="1:13" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1088" s="6"/>
+      <c r="B1088" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="C1088" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1088" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1088" s="2">
+        <v>0</v>
+      </c>
+      <c r="F1088" s="2">
+        <v>4430000</v>
+      </c>
+      <c r="G1088" s="2">
+        <v>4470000</v>
+      </c>
+      <c r="H1088" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="I1088" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1088" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1088" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1088" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="M1088" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1089" spans="1:13" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1089" s="6"/>
+      <c r="B1089" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="C1089" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1089" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E1089" s="2">
+        <v>51</v>
+      </c>
+      <c r="F1089" s="2">
+        <v>2630000</v>
+      </c>
+      <c r="G1089" s="2">
+        <v>2730000</v>
+      </c>
+      <c r="H1089" s="2" t="s">
+        <v>246</v>
+      </c>
+      <c r="I1089" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1089" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1089" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1089" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="M1089" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1090" spans="1:13" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1090" s="6"/>
+      <c r="B1090" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="C1090" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1090" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E1090" s="2">
+        <v>119</v>
+      </c>
+      <c r="F1090" s="2">
+        <v>6180000</v>
+      </c>
+      <c r="G1090" s="2">
+        <v>6110000</v>
+      </c>
+      <c r="H1090" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="I1090" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1090" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1090" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1090" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="M1090" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1091" spans="1:13" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1091" s="6"/>
+      <c r="B1091" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="C1091" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1091" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E1091" s="2">
+        <v>0</v>
+      </c>
+      <c r="F1091" s="2">
+        <v>170000</v>
+      </c>
+      <c r="G1091" s="2">
+        <v>170000</v>
+      </c>
+      <c r="H1091" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="I1091" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1091" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="K1091" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1091" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="M1091" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1092" spans="1:13" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1092" s="6"/>
+      <c r="B1092" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="C1092" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1092" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E1092" s="2">
+        <v>127</v>
+      </c>
+      <c r="F1092" s="2">
+        <v>6530000</v>
+      </c>
+      <c r="G1092" s="2">
+        <v>6400000</v>
+      </c>
+      <c r="H1092" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="I1092" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1092" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1092" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1092" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="M1092" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1093" spans="1:13" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1093" s="6"/>
+      <c r="B1093" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="C1093" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1093" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E1093" s="2">
+        <v>69</v>
+      </c>
+      <c r="F1093" s="2">
+        <v>4770000</v>
+      </c>
+      <c r="G1093" s="2">
+        <v>4810000</v>
+      </c>
+      <c r="H1093" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="I1093" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1093" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1093" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1093" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="M1093" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1094" spans="1:13" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1094" s="6"/>
+      <c r="B1094" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="C1094" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1094" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1094" s="2">
+        <v>68</v>
+      </c>
+      <c r="F1094" s="2">
+        <v>4360000</v>
+      </c>
+      <c r="G1094" s="2">
+        <v>4400000</v>
+      </c>
+      <c r="H1094" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="I1094" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1094" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="K1094" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1094" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="M1094" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1095" spans="1:13" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1095" s="6"/>
+      <c r="B1095" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="C1095" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1095" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="E1095" s="2">
+        <v>81</v>
+      </c>
+      <c r="F1095" s="2">
+        <v>1550000</v>
+      </c>
+      <c r="G1095" s="2">
+        <v>1560000</v>
+      </c>
+      <c r="H1095" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="I1095" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1095" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1095" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1095" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="M1095" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1096" spans="1:13" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1096" s="6"/>
+      <c r="B1096" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="C1096" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1096" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="E1096" s="2">
+        <v>123</v>
+      </c>
+      <c r="F1096" s="2">
+        <v>5340000</v>
+      </c>
+      <c r="G1096" s="2">
+        <v>5350000</v>
+      </c>
+      <c r="H1096" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="I1096" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1096" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1096" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1096" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="M1096" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1097" spans="1:13" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1097" s="6"/>
+      <c r="B1097" s="2" t="s">
+        <v>289</v>
+      </c>
+      <c r="C1097" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1097" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="E1097" s="2">
+        <v>128</v>
+      </c>
+      <c r="F1097" s="2">
+        <v>4690000</v>
+      </c>
+      <c r="G1097" s="2">
+        <v>4680000</v>
+      </c>
+      <c r="H1097" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="I1097" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1097" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1097" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1097" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="M1097" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1098" spans="1:13" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1098" s="6"/>
+      <c r="B1098" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="C1098" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1098" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="E1098" s="2">
+        <v>109</v>
+      </c>
+      <c r="F1098" s="2">
+        <v>3900000</v>
+      </c>
+      <c r="G1098" s="2">
+        <v>3820000</v>
+      </c>
+      <c r="H1098" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="I1098" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1098" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1098" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1098" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="M1098" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1099" spans="1:13" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1099" s="6"/>
+      <c r="B1099" s="2" t="s">
+        <v>290</v>
+      </c>
+      <c r="C1099" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1099" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1099" s="2">
+        <v>0</v>
+      </c>
+      <c r="F1099" s="2">
+        <v>160000</v>
+      </c>
+      <c r="G1099" s="2">
+        <v>160000</v>
+      </c>
+      <c r="H1099" s="2" t="s">
+        <v>291</v>
+      </c>
+      <c r="I1099" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1099" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="K1099" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1099" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1099" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1100" spans="1:13" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1100" s="6"/>
+      <c r="B1100" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="C1100" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1100" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E1100" s="2">
+        <v>16</v>
+      </c>
+      <c r="F1100" s="2">
+        <v>460000</v>
+      </c>
+      <c r="G1100" s="2">
+        <v>460000</v>
+      </c>
+      <c r="H1100" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="I1100" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1100" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1100" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1100" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="M1100" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1101" spans="1:13" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1101" s="6"/>
+      <c r="B1101" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="C1101" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1101" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E1101" s="2">
+        <v>0</v>
+      </c>
+      <c r="F1101" s="2">
+        <v>1970000</v>
+      </c>
+      <c r="G1101" s="2">
+        <v>1960000</v>
+      </c>
+      <c r="H1101" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="I1101" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1101" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="K1101" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1101" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="M1101" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1102" spans="1:13" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1102" s="6"/>
+      <c r="B1102" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="C1102" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1102" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="E1102" s="2">
+        <v>12</v>
+      </c>
+      <c r="F1102" s="2">
+        <v>640000</v>
+      </c>
+      <c r="G1102" s="2">
+        <v>640000</v>
+      </c>
+      <c r="H1102" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="I1102" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1102" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1102" s="2">
+        <v>1</v>
+      </c>
+      <c r="L1102" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="M1102" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1103" spans="1:13" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1103" s="6"/>
+      <c r="B1103" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="C1103" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1103" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E1103" s="2">
+        <v>0</v>
+      </c>
+      <c r="F1103" s="2">
+        <v>10640000</v>
+      </c>
+      <c r="G1103" s="2">
+        <v>11300000</v>
+      </c>
+      <c r="H1103" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="I1103" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1103" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="K1103" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1103" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="M1103" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1104" spans="1:13" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1104" s="6"/>
+      <c r="B1104" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="C1104" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1104" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E1104" s="2">
+        <v>118</v>
+      </c>
+      <c r="F1104" s="2">
+        <v>6680000</v>
+      </c>
+      <c r="G1104" s="2">
+        <v>6530000</v>
+      </c>
+      <c r="H1104" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="I1104" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1104" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1104" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1104" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="M1104" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1105" spans="1:13" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1105" s="6"/>
+      <c r="B1105" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="C1105" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1105" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E1105" s="2">
+        <v>30</v>
+      </c>
+      <c r="F1105" s="2">
+        <v>2500000</v>
+      </c>
+      <c r="G1105" s="2">
+        <v>2630000</v>
+      </c>
+      <c r="H1105" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="I1105" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1105" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1105" s="2">
+        <v>1</v>
+      </c>
+      <c r="L1105" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1105" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1106" spans="1:13" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1106" s="6"/>
+      <c r="B1106" s="2" t="s">
+        <v>260</v>
+      </c>
+      <c r="C1106" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1106" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="E1106" s="2">
+        <v>0</v>
+      </c>
+      <c r="F1106" s="2">
+        <v>260000</v>
+      </c>
+      <c r="G1106" s="2">
+        <v>260000</v>
+      </c>
+      <c r="H1106" s="2" t="s">
+        <v>261</v>
+      </c>
+      <c r="I1106" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1106" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1106" s="2">
+        <v>4</v>
+      </c>
+      <c r="L1106" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1106" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1107" spans="1:13" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1107" s="6"/>
+      <c r="B1107" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="C1107" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1107" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E1107" s="2">
+        <v>54</v>
+      </c>
+      <c r="F1107" s="2">
+        <v>2300000</v>
+      </c>
+      <c r="G1107" s="2">
+        <v>2300000</v>
+      </c>
+      <c r="H1107" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="I1107" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1107" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1107" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1107" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="M1107" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1108" spans="1:13" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1108" s="6"/>
+      <c r="B1108" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="C1108" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1108" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E1108" s="2">
+        <v>89</v>
+      </c>
+      <c r="F1108" s="2">
+        <v>8520000</v>
+      </c>
+      <c r="G1108" s="2">
+        <v>8460000</v>
+      </c>
+      <c r="H1108" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="I1108" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1108" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1108" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1108" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="M1108" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1109" spans="1:13" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1109" s="6"/>
+      <c r="B1109" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="C1109" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1109" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="E1109" s="2">
+        <v>130</v>
+      </c>
+      <c r="F1109" s="2">
+        <v>12090000</v>
+      </c>
+      <c r="G1109" s="2">
+        <v>12150000</v>
+      </c>
+      <c r="H1109" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="I1109" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1109" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="K1109" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1109" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="M1109" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1110" spans="1:13" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1110" s="6"/>
+      <c r="B1110" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="C1110" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1110" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1110" s="2">
+        <v>0</v>
+      </c>
+      <c r="F1110" s="2">
+        <v>1920000</v>
+      </c>
+      <c r="G1110" s="2">
+        <v>1900000</v>
+      </c>
+      <c r="H1110" s="2" t="s">
+        <v>241</v>
+      </c>
+      <c r="I1110" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1110" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1110" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1110" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="M1110" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1111" spans="1:13" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1111" s="6"/>
+      <c r="B1111" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="C1111" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1111" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1111" s="2">
+        <v>91</v>
+      </c>
+      <c r="F1111" s="2">
+        <v>8730000</v>
+      </c>
+      <c r="G1111" s="2">
+        <v>8660000</v>
+      </c>
+      <c r="H1111" s="2" t="s">
+        <v>264</v>
+      </c>
+      <c r="I1111" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1111" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1111" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1111" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="M1111" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1112" spans="1:13" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1112" s="6"/>
+      <c r="B1112" s="2" t="s">
+        <v>292</v>
+      </c>
+      <c r="C1112" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1112" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="E1112" s="2">
+        <v>30</v>
+      </c>
+      <c r="F1112" s="2">
+        <v>880000</v>
+      </c>
+      <c r="G1112" s="2">
+        <v>870000</v>
+      </c>
+      <c r="H1112" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="I1112" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1112" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1112" s="2">
+        <v>1</v>
+      </c>
+      <c r="L1112" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1112" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1113" spans="1:13" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1113" s="6"/>
+      <c r="B1113" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="C1113" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1113" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="E1113" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1113" s="2">
+        <v>290000</v>
+      </c>
+      <c r="G1113" s="2">
+        <v>290000</v>
+      </c>
+      <c r="H1113" s="2" t="s">
+        <v>244</v>
+      </c>
+      <c r="I1113" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1113" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="K1113" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1113" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="M1113" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1114" spans="1:13" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1114" s="6"/>
+      <c r="B1114" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="C1114" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1114" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="E1114" s="2">
+        <v>108</v>
+      </c>
+      <c r="F1114" s="2">
+        <v>3200000</v>
+      </c>
+      <c r="G1114" s="2">
+        <v>3170000</v>
+      </c>
+      <c r="H1114" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="I1114" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1114" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1114" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1114" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="M1114" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1115" spans="1:13" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1115" s="6"/>
+      <c r="B1115" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="C1115" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1115" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="E1115" s="2">
+        <v>112</v>
+      </c>
+      <c r="F1115" s="2">
+        <v>4120000</v>
+      </c>
+      <c r="G1115" s="2">
+        <v>4110000</v>
+      </c>
+      <c r="H1115" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="I1115" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="J1115" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1115" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1115" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="M1115" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1116" spans="1:13" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1116" s="6"/>
+      <c r="B1116" s="2" t="s">
+        <v>278</v>
+      </c>
+      <c r="C1116" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1116" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E1116" s="2">
+        <v>136</v>
+      </c>
+      <c r="F1116" s="2">
+        <v>7340000</v>
+      </c>
+      <c r="G1116" s="2">
+        <v>7330000</v>
+      </c>
+      <c r="H1116" s="2" t="s">
+        <v>279</v>
+      </c>
+      <c r="I1116" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1116" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1116" s="2">
+        <v>1</v>
+      </c>
+      <c r="L1116" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1116" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1117" spans="1:13" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1117" s="6"/>
+      <c r="B1117" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="C1117" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1117" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="E1117" s="2">
+        <v>90</v>
+      </c>
+      <c r="F1117" s="2">
+        <v>3610000</v>
+      </c>
+      <c r="G1117" s="2">
+        <v>3590000</v>
+      </c>
+      <c r="H1117" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="I1117" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1117" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1117" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1117" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="M1117" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1118" spans="1:13" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1118" s="6"/>
+      <c r="B1118" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="C1118" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1118" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="E1118" s="2">
+        <v>15</v>
+      </c>
+      <c r="F1118" s="2">
+        <v>390000</v>
+      </c>
+      <c r="G1118" s="2">
+        <v>390000</v>
+      </c>
+      <c r="H1118" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="I1118" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1118" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1118" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1118" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="M1118" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1119" spans="1:13" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1119" s="6"/>
+      <c r="B1119" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="C1119" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1119" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="E1119" s="2">
+        <v>58</v>
+      </c>
+      <c r="F1119" s="2">
+        <v>1310000</v>
+      </c>
+      <c r="G1119" s="2">
+        <v>1300000</v>
+      </c>
+      <c r="H1119" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="I1119" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1119" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1119" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1119" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="M1119" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1120" spans="1:13" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1120" s="6"/>
+      <c r="B1120" s="2" t="s">
+        <v>293</v>
+      </c>
+      <c r="C1120" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1120" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="E1120" s="2">
+        <v>48</v>
+      </c>
+      <c r="F1120" s="2">
+        <v>1660000</v>
+      </c>
+      <c r="G1120" s="2">
+        <v>1650000</v>
+      </c>
+      <c r="H1120" s="2" t="s">
+        <v>246</v>
+      </c>
+      <c r="I1120" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1120" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1120" s="2">
+        <v>5</v>
+      </c>
+      <c r="L1120" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1120" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1121" spans="1:13" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1121" s="6"/>
+      <c r="B1121" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="C1121" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1121" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E1121" s="2">
+        <v>77</v>
+      </c>
+      <c r="F1121" s="2">
+        <v>4640000</v>
+      </c>
+      <c r="G1121" s="2">
+        <v>4670000</v>
+      </c>
+      <c r="H1121" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="I1121" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1121" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1121" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1121" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="M1121" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1122" spans="1:13" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1122" s="6"/>
+      <c r="B1122" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="C1122" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1122" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="E1122" s="2">
+        <v>4</v>
+      </c>
+      <c r="F1122" s="2">
+        <v>420000</v>
+      </c>
+      <c r="G1122" s="2">
+        <v>420000</v>
+      </c>
+      <c r="H1122" s="2" t="s">
+        <v>244</v>
+      </c>
+      <c r="I1122" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1122" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="K1122" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1122" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="M1122" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1123" spans="1:13" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1123" s="6"/>
+      <c r="B1123" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="C1123" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1123" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E1123" s="2">
+        <v>47</v>
+      </c>
+      <c r="F1123" s="2">
+        <v>1410000</v>
+      </c>
+      <c r="G1123" s="2">
+        <v>1380000</v>
+      </c>
+      <c r="H1123" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="I1123" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1123" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1123" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1123" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="M1123" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1124" spans="1:13" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1124" s="6"/>
+      <c r="B1124" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="C1124" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1124" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E1124" s="2">
+        <v>156</v>
+      </c>
+      <c r="F1124" s="2">
+        <v>6840000</v>
+      </c>
+      <c r="G1124" s="2">
+        <v>6760000</v>
+      </c>
+      <c r="H1124" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="I1124" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1124" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1124" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1124" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="M1124" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1125" spans="1:13" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1125" s="6"/>
+      <c r="B1125" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="C1125" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1125" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="E1125" s="2">
+        <v>29</v>
+      </c>
+      <c r="F1125" s="2">
+        <v>850000</v>
+      </c>
+      <c r="G1125" s="2">
+        <v>840000</v>
+      </c>
+      <c r="H1125" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="I1125" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1125" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1125" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1125" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="M1125" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1126" spans="1:13" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1126" s="6"/>
+      <c r="B1126" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="C1126" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1126" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E1126" s="2">
+        <v>102</v>
+      </c>
+      <c r="F1126" s="2">
+        <v>2750000</v>
+      </c>
+      <c r="G1126" s="2">
+        <v>2730000</v>
+      </c>
+      <c r="H1126" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="I1126" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1126" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1126" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1126" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="M1126" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1127" spans="1:13" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1127" s="6"/>
+      <c r="B1127" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="C1127" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1127" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="E1127" s="2">
+        <v>19</v>
+      </c>
+      <c r="F1127" s="2">
+        <v>910000</v>
+      </c>
+      <c r="G1127" s="2">
+        <v>900000</v>
+      </c>
+      <c r="H1127" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="I1127" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1127" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1127" s="2">
+        <v>1</v>
+      </c>
+      <c r="L1127" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1127" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1128" spans="1:13" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1128" s="6"/>
+      <c r="B1128" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="C1128" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1128" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E1128" s="2">
+        <v>11</v>
+      </c>
+      <c r="F1128" s="2">
+        <v>2870000</v>
+      </c>
+      <c r="G1128" s="2">
+        <v>2940000</v>
+      </c>
+      <c r="H1128" s="2" t="s">
+        <v>265</v>
+      </c>
+      <c r="I1128" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1128" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="K1128" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1128" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="M1128" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1129" spans="1:13" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1129" s="6"/>
+      <c r="B1129" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="C1129" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1129" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E1129" s="2">
+        <v>40</v>
+      </c>
+      <c r="F1129" s="2">
+        <v>2390000</v>
+      </c>
+      <c r="G1129" s="2">
+        <v>2360000</v>
+      </c>
+      <c r="H1129" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="I1129" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1129" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1129" s="2">
+        <v>1</v>
+      </c>
+      <c r="L1129" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="M1129" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1130" spans="1:13" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1130" s="6"/>
+      <c r="B1130" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="C1130" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1130" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="E1130" s="2">
+        <v>17</v>
+      </c>
+      <c r="F1130" s="2">
+        <v>1400000</v>
+      </c>
+      <c r="G1130" s="2">
+        <v>1420000</v>
+      </c>
+      <c r="H1130" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="I1130" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1130" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1130" s="2">
+        <v>1</v>
+      </c>
+      <c r="L1130" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="M1130" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1131" spans="1:13" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1131" s="6"/>
+      <c r="B1131" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="C1131" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1131" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="E1131" s="2">
+        <v>0</v>
+      </c>
+      <c r="F1131" s="2">
+        <v>160000</v>
+      </c>
+      <c r="G1131" s="2">
+        <v>160000</v>
+      </c>
+      <c r="H1131" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="I1131" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1131" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="K1131" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1131" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1131" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1132" spans="1:13" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1132" s="6"/>
+      <c r="B1132" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="C1132" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1132" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="E1132" s="2">
+        <v>0</v>
+      </c>
+      <c r="F1132" s="2">
+        <v>3650000</v>
+      </c>
+      <c r="G1132" s="2">
+        <v>3610000</v>
+      </c>
+      <c r="H1132" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="I1132" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1132" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="K1132" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1132" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="M1132" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1133" spans="1:13" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1133" s="6"/>
+      <c r="B1133" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="C1133" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1133" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="E1133" s="2">
+        <v>0</v>
+      </c>
+      <c r="F1133" s="2">
+        <v>190000</v>
+      </c>
+      <c r="G1133" s="2">
+        <v>190000</v>
+      </c>
+      <c r="H1133" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="I1133" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1133" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="K1133" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1133" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1133" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1134" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1134" s="6"/>
+      <c r="B1134" s="2" t="s">
+        <v>272</v>
+      </c>
+      <c r="C1134" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1134" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="E1134" s="2">
+        <v>0</v>
+      </c>
+      <c r="F1134" s="2">
+        <v>3520000</v>
+      </c>
+      <c r="G1134" s="2">
+        <v>3400000</v>
+      </c>
+      <c r="H1134" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="I1134" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1134" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="K1134" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1134" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1134" s="7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="1135" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="M1135" s="7"/>
     </row>
   </sheetData>
   <autoFilter ref="B1:M1" xr:uid="{93EB6F54-7766-4759-97DF-03549A275A7C}">
@@ -40972,8 +44488,97 @@
     <hyperlink ref="B964" r:id="rId427" display="https://www.com-analytics.de/player/34146" xr:uid="{6D366095-4485-4799-820E-0163C666B073}"/>
     <hyperlink ref="B965" r:id="rId428" display="https://www.com-analytics.de/player/34148" xr:uid="{41264995-04B2-4496-A841-8876A9A7B88E}"/>
     <hyperlink ref="B966" r:id="rId429" display="https://www.com-analytics.de/player/34187" xr:uid="{6B55E76B-D339-42F6-AC79-CB79A92F7E6E}"/>
+    <hyperlink ref="B1046" r:id="rId430" display="https://www.com-analytics.de/player/30755" xr:uid="{B0FFC3B6-B77F-4227-944F-07B23F45EFA9}"/>
+    <hyperlink ref="B1047" r:id="rId431" display="https://www.com-analytics.de/player/31419" xr:uid="{8386018F-208B-472E-A6DD-53190B9BF445}"/>
+    <hyperlink ref="B1048" r:id="rId432" display="https://www.com-analytics.de/player/31846" xr:uid="{8CAF91C6-74F7-4630-A075-65300CC21E77}"/>
+    <hyperlink ref="B1049" r:id="rId433" display="https://www.com-analytics.de/player/31910" xr:uid="{58FA4847-C907-4DAF-810B-16DA9826BFB7}"/>
+    <hyperlink ref="B1050" r:id="rId434" display="https://www.com-analytics.de/player/31932" xr:uid="{4CE92407-DE5F-4E93-8B82-8A8F4BF37D8F}"/>
+    <hyperlink ref="B1051" r:id="rId435" display="https://www.com-analytics.de/player/31958" xr:uid="{E90F4231-2B27-45C1-9261-B5ADFA8B5FB1}"/>
+    <hyperlink ref="B1052" r:id="rId436" display="https://www.com-analytics.de/player/32080" xr:uid="{8ABBB07B-7425-47EC-97D9-4925AF302F4F}"/>
+    <hyperlink ref="B1053" r:id="rId437" display="https://www.com-analytics.de/player/32122" xr:uid="{073A333A-069F-4C44-BE6B-376A62E7BAF0}"/>
+    <hyperlink ref="B1054" r:id="rId438" display="https://www.com-analytics.de/player/32310" xr:uid="{77084502-ABE8-4536-A329-056A25448C0B}"/>
+    <hyperlink ref="B1055" r:id="rId439" display="https://www.com-analytics.de/player/32364" xr:uid="{BE70D4EF-EC97-47AE-8374-D2E5CDE13296}"/>
+    <hyperlink ref="B1056" r:id="rId440" display="https://www.com-analytics.de/player/32398" xr:uid="{5016B014-CA6F-4E0B-A9B4-7CC7EEC8FEE8}"/>
+    <hyperlink ref="B1057" r:id="rId441" display="https://www.com-analytics.de/player/32472" xr:uid="{32932586-0995-4BDD-A058-F4B06AB1A829}"/>
+    <hyperlink ref="B1058" r:id="rId442" display="https://www.com-analytics.de/player/32509" xr:uid="{CD183843-15D6-4661-935E-0DD05B639C42}"/>
+    <hyperlink ref="B1059" r:id="rId443" display="https://www.com-analytics.de/player/32553" xr:uid="{7D343D60-BE89-4528-ACE7-876B6C15D57D}"/>
+    <hyperlink ref="B1060" r:id="rId444" display="https://www.com-analytics.de/player/32575" xr:uid="{25C1DE99-9D80-4F2F-8E3E-D31BE62DD265}"/>
+    <hyperlink ref="B1061" r:id="rId445" display="https://www.com-analytics.de/player/32579" xr:uid="{73ABBBB9-78BF-442A-9A66-A2EA144FD3F8}"/>
+    <hyperlink ref="B1062" r:id="rId446" display="https://www.com-analytics.de/player/32603" xr:uid="{1C57847F-6CCE-4E77-828D-9DCDCFF814F2}"/>
+    <hyperlink ref="B1063" r:id="rId447" display="https://www.com-analytics.de/player/32629" xr:uid="{1565101F-76AF-47F7-9A37-655F9A28F485}"/>
+    <hyperlink ref="B1064" r:id="rId448" display="https://www.com-analytics.de/player/32630" xr:uid="{45E4510D-DB3B-4DBB-97C1-3918E12E4B20}"/>
+    <hyperlink ref="B1065" r:id="rId449" display="https://www.com-analytics.de/player/32633" xr:uid="{4A99EF4F-1E9F-4176-93AF-60AB42C13C27}"/>
+    <hyperlink ref="B1066" r:id="rId450" display="https://www.com-analytics.de/player/32636" xr:uid="{4D6CA489-C7DA-40ED-B1AF-1D8558576F66}"/>
+    <hyperlink ref="B1067" r:id="rId451" display="https://www.com-analytics.de/player/32738" xr:uid="{A63EB659-8B5E-4612-B7C7-4128F9182F01}"/>
+    <hyperlink ref="B1068" r:id="rId452" display="https://www.com-analytics.de/player/32744" xr:uid="{90DAC7E3-D4EF-4FAB-AE2C-4CAA9E083B7D}"/>
+    <hyperlink ref="B1069" r:id="rId453" display="https://www.com-analytics.de/player/32754" xr:uid="{F3DF93A7-B5CF-4AC5-84C7-E6A85FFEB67A}"/>
+    <hyperlink ref="B1070" r:id="rId454" display="https://www.com-analytics.de/player/32756" xr:uid="{2BF42AC4-572F-4742-92BB-4B439A7F7ED5}"/>
+    <hyperlink ref="B1071" r:id="rId455" display="https://www.com-analytics.de/player/32787" xr:uid="{4D651536-12A6-4C38-B65F-973AEF94C6F9}"/>
+    <hyperlink ref="B1072" r:id="rId456" display="https://www.com-analytics.de/player/32841" xr:uid="{4E88EBF8-7C05-44AE-9CC4-E1A2AA1C3635}"/>
+    <hyperlink ref="B1073" r:id="rId457" display="https://www.com-analytics.de/player/32877" xr:uid="{A8E4FC38-0313-43CB-AFE1-ED190819EF9C}"/>
+    <hyperlink ref="B1074" r:id="rId458" display="https://www.com-analytics.de/player/32931" xr:uid="{3BC17B98-FF4A-4FE4-A4E7-49DCA9C1A256}"/>
+    <hyperlink ref="B1075" r:id="rId459" display="https://www.com-analytics.de/player/32948" xr:uid="{D1F98622-F473-47C7-8F64-5780D321712F}"/>
+    <hyperlink ref="B1076" r:id="rId460" display="https://www.com-analytics.de/player/32977" xr:uid="{2FBAC77F-F4C1-4322-9E5E-8B0FFFAC0CF4}"/>
+    <hyperlink ref="B1077" r:id="rId461" display="https://www.com-analytics.de/player/33070" xr:uid="{FCD46820-C12A-4166-B999-D6B490807A25}"/>
+    <hyperlink ref="B1078" r:id="rId462" display="https://www.com-analytics.de/player/33096" xr:uid="{8046DE26-1F8B-41D0-9753-6B77620B64A8}"/>
+    <hyperlink ref="B1079" r:id="rId463" display="https://www.com-analytics.de/player/33105" xr:uid="{ADF94AB4-61B8-4780-AC12-64055D52B341}"/>
+    <hyperlink ref="B1080" r:id="rId464" display="https://www.com-analytics.de/player/33109" xr:uid="{6782FCF7-4CEB-4AF3-9F1F-4E5BF2C22544}"/>
+    <hyperlink ref="B1081" r:id="rId465" display="https://www.com-analytics.de/player/33133" xr:uid="{304A4B82-011D-43BD-B4C2-56772EB62FC1}"/>
+    <hyperlink ref="B1082" r:id="rId466" display="https://www.com-analytics.de/player/33156" xr:uid="{5C57AEED-309C-4375-AFFD-B86A082194A7}"/>
+    <hyperlink ref="B1083" r:id="rId467" display="https://www.com-analytics.de/player/33157" xr:uid="{1FDB6A19-39C8-4872-BFA5-0185458226B2}"/>
+    <hyperlink ref="B1084" r:id="rId468" display="https://www.com-analytics.de/player/33236" xr:uid="{1E2D8F80-9781-4EF3-B5E3-92211F928DA9}"/>
+    <hyperlink ref="B1085" r:id="rId469" display="https://www.com-analytics.de/player/33296" xr:uid="{EFDA8CB1-CA43-4636-8311-8B7961621E28}"/>
+    <hyperlink ref="B1086" r:id="rId470" display="https://www.com-analytics.de/player/33313" xr:uid="{18AD819C-16EF-4721-B6A7-022B610E0102}"/>
+    <hyperlink ref="B1087" r:id="rId471" display="https://www.com-analytics.de/player/33335" xr:uid="{0B96B4A1-08A8-4CFE-B7FB-9179F0F9F3F2}"/>
+    <hyperlink ref="B1088" r:id="rId472" display="https://www.com-analytics.de/player/33356" xr:uid="{8F8F55C3-73EE-418E-A180-EAF05A91AAE9}"/>
+    <hyperlink ref="B1089" r:id="rId473" display="https://www.com-analytics.de/player/33364" xr:uid="{F965E591-A7EF-4E67-8DE1-791F14A0C546}"/>
+    <hyperlink ref="B1090" r:id="rId474" display="https://www.com-analytics.de/player/33383" xr:uid="{E619F695-99E8-4A6A-ADCE-E9F58C89731D}"/>
+    <hyperlink ref="B1091" r:id="rId475" display="https://www.com-analytics.de/player/33397" xr:uid="{25071E93-9F0E-4F36-86EB-704A73EA4349}"/>
+    <hyperlink ref="B1092" r:id="rId476" display="https://www.com-analytics.de/player/33409" xr:uid="{F47981E6-231B-41C7-8DE9-E074662F69BC}"/>
+    <hyperlink ref="B1093" r:id="rId477" display="https://www.com-analytics.de/player/33514" xr:uid="{957FDB37-1D0D-4C8C-BEF4-68EC5ED3F4B7}"/>
+    <hyperlink ref="B1094" r:id="rId478" display="https://www.com-analytics.de/player/33547" xr:uid="{877AC8EF-5874-4DDD-BC6E-4624F5DB5985}"/>
+    <hyperlink ref="B1095" r:id="rId479" display="https://www.com-analytics.de/player/33550" xr:uid="{4DE94E2C-B767-409E-851D-E4BCAB9C6D05}"/>
+    <hyperlink ref="B1096" r:id="rId480" display="https://www.com-analytics.de/player/33552" xr:uid="{3243CC70-5696-418B-B480-5E47EE74FD0C}"/>
+    <hyperlink ref="B1097" r:id="rId481" display="https://www.com-analytics.de/player/33577" xr:uid="{9CB34097-A966-4286-858D-814A86DCCDD4}"/>
+    <hyperlink ref="B1098" r:id="rId482" display="https://www.com-analytics.de/player/33609" xr:uid="{EB514D1F-5885-40DC-8FA3-25299A01C4C4}"/>
+    <hyperlink ref="B1099" r:id="rId483" display="https://www.com-analytics.de/player/33615" xr:uid="{A1880EB6-6CF2-4CB4-8CB7-63509137F936}"/>
+    <hyperlink ref="B1100" r:id="rId484" display="https://www.com-analytics.de/player/33678" xr:uid="{5DEF044A-E702-498E-B7A8-634A776058C0}"/>
+    <hyperlink ref="B1101" r:id="rId485" display="https://www.com-analytics.de/player/33696" xr:uid="{98A598D2-2854-4CA3-B83A-FBA1A200542E}"/>
+    <hyperlink ref="B1102" r:id="rId486" display="https://www.com-analytics.de/player/33718" xr:uid="{BDB7D5B4-05AA-44CF-8AD2-81BA0F1D3285}"/>
+    <hyperlink ref="B1103" r:id="rId487" display="https://www.com-analytics.de/player/33744" xr:uid="{23885634-3738-48A2-AD11-97DF53052028}"/>
+    <hyperlink ref="B1104" r:id="rId488" display="https://www.com-analytics.de/player/33782" xr:uid="{4649082F-B540-4322-A373-40E0052EC182}"/>
+    <hyperlink ref="B1105" r:id="rId489" display="https://www.com-analytics.de/player/33783" xr:uid="{8F567C4F-8C1B-4732-BC8D-DC8663073113}"/>
+    <hyperlink ref="B1106" r:id="rId490" display="https://www.com-analytics.de/player/33812" xr:uid="{9B27461B-BB58-45F8-B3A5-9D73DA9357BA}"/>
+    <hyperlink ref="B1107" r:id="rId491" display="https://www.com-analytics.de/player/33815" xr:uid="{C0BAF3BD-1B1D-4F6B-8343-DF2AB55507B4}"/>
+    <hyperlink ref="B1108" r:id="rId492" display="https://www.com-analytics.de/player/33827" xr:uid="{FCB2F52A-3536-494E-A44E-BEB2A5D3C245}"/>
+    <hyperlink ref="B1109" r:id="rId493" display="https://www.com-analytics.de/player/33832" xr:uid="{BF353C95-EFA3-48E6-B92F-B6BD66E66228}"/>
+    <hyperlink ref="B1110" r:id="rId494" display="https://www.com-analytics.de/player/33848" xr:uid="{C53C71E8-8CB5-4D6F-B243-EDCDD6A0C81E}"/>
+    <hyperlink ref="B1111" r:id="rId495" display="https://www.com-analytics.de/player/33854" xr:uid="{296900CA-745A-4E27-81B7-3471D09EA7A4}"/>
+    <hyperlink ref="B1112" r:id="rId496" display="https://www.com-analytics.de/player/33882" xr:uid="{BC163EDD-250F-48CC-9809-3E540E8C88EC}"/>
+    <hyperlink ref="B1113" r:id="rId497" display="https://www.com-analytics.de/player/33905" xr:uid="{71A948AF-9004-46B6-A77E-A6E963632398}"/>
+    <hyperlink ref="B1114" r:id="rId498" display="https://www.com-analytics.de/player/33948" xr:uid="{A1217C8A-55F5-4B7E-B67B-8FE39221A118}"/>
+    <hyperlink ref="B1115" r:id="rId499" display="https://www.com-analytics.de/player/33950" xr:uid="{CCC992F9-B8F0-4177-9BD5-C5E6DCE037F3}"/>
+    <hyperlink ref="B1116" r:id="rId500" display="https://www.com-analytics.de/player/33992" xr:uid="{825CEF13-B07C-41A4-98E4-C3E3C10B8B76}"/>
+    <hyperlink ref="B1117" r:id="rId501" display="https://www.com-analytics.de/player/33995" xr:uid="{A5B6FDEA-2C88-4845-B8ED-B09FD6D72032}"/>
+    <hyperlink ref="B1118" r:id="rId502" display="https://www.com-analytics.de/player/33999" xr:uid="{0E27C336-2D91-40DE-9D62-9CD8EC0D7F16}"/>
+    <hyperlink ref="B1119" r:id="rId503" display="https://www.com-analytics.de/player/34001" xr:uid="{179B37F7-1D00-4A68-A80E-E97D2046A5E1}"/>
+    <hyperlink ref="B1120" r:id="rId504" display="https://www.com-analytics.de/player/34006" xr:uid="{036A1A8F-7C55-49F7-9D89-154A27150793}"/>
+    <hyperlink ref="B1121" r:id="rId505" display="https://www.com-analytics.de/player/34008" xr:uid="{8F276541-95AA-475E-8864-CEE5B8A5A255}"/>
+    <hyperlink ref="B1122" r:id="rId506" display="https://www.com-analytics.de/player/34011" xr:uid="{1E45224E-EA63-4149-960C-823E9DE65323}"/>
+    <hyperlink ref="B1123" r:id="rId507" display="https://www.com-analytics.de/player/34019" xr:uid="{C21D6BBB-1307-442A-B3C8-E1E35C5A405E}"/>
+    <hyperlink ref="B1124" r:id="rId508" display="https://www.com-analytics.de/player/34025" xr:uid="{0BF9F279-3094-43F5-B7EF-E79515D825A4}"/>
+    <hyperlink ref="B1125" r:id="rId509" display="https://www.com-analytics.de/player/34035" xr:uid="{E29984F5-0F89-4188-9B4B-C9EC42EA7A72}"/>
+    <hyperlink ref="B1126" r:id="rId510" display="https://www.com-analytics.de/player/34044" xr:uid="{5AA058BD-284F-4A20-8C47-DD924002D2FC}"/>
+    <hyperlink ref="B1127" r:id="rId511" display="https://www.com-analytics.de/player/34050" xr:uid="{DBD2C17E-BFE8-40EC-8FD0-09086C35A9F8}"/>
+    <hyperlink ref="B1128" r:id="rId512" display="https://www.com-analytics.de/player/34096" xr:uid="{B6CD9502-BD82-4B3A-B66B-031BF9D3F3D5}"/>
+    <hyperlink ref="B1129" r:id="rId513" display="https://www.com-analytics.de/player/34109" xr:uid="{91B389C9-525F-4264-B4F9-C356E18DCB87}"/>
+    <hyperlink ref="B1130" r:id="rId514" display="https://www.com-analytics.de/player/34116" xr:uid="{A80DCB19-FC15-4F57-9960-CF9B5BAAEB48}"/>
+    <hyperlink ref="B1131" r:id="rId515" display="https://www.com-analytics.de/player/34126" xr:uid="{86467537-CA43-41A4-937B-75925D7C7607}"/>
+    <hyperlink ref="B1132" r:id="rId516" display="https://www.com-analytics.de/player/34148" xr:uid="{F0E18F02-56BE-4BD4-A4AE-A50E27943A12}"/>
+    <hyperlink ref="B1133" r:id="rId517" display="https://www.com-analytics.de/player/34162" xr:uid="{500CBE5D-421A-4406-A639-70907E3EC3EC}"/>
+    <hyperlink ref="B1134" r:id="rId518" display="https://www.com-analytics.de/player/34187" xr:uid="{A98B63D0-4871-4962-94BB-899FCB9DFCA2}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" r:id="rId430"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" r:id="rId519"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Automatisches Update TM + Transfers - 14.06.2025 08:35
</commit_message>
<xml_diff>
--- a/TM_all.xlsx
+++ b/TM_all.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/aecf56309e6168f4/Documents/comunio/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="234" documentId="8_{B00F7E9F-5C85-449B-834E-0179FBCEE2D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{51C20D1E-0DF0-489C-83F1-A6D45CB1609D}"/>
+  <xr:revisionPtr revIDLastSave="239" documentId="8_{B00F7E9F-5C85-449B-834E-0179FBCEE2D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E2CB34A4-E516-4A1A-8BA5-8CA4166C45EF}"/>
   <bookViews>
     <workbookView xWindow="6660" yWindow="2700" windowWidth="28800" windowHeight="15370" xr2:uid="{607DE709-F91E-4262-9941-1066BBEC319E}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7987" uniqueCount="295">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8675" uniqueCount="302">
   <si>
     <t>Spieler</t>
   </si>
@@ -925,6 +925,27 @@
   <si>
     <t>13.06.2025</t>
   </si>
+  <si>
+    <t>Klostermann</t>
+  </si>
+  <si>
+    <t>N. Schlotterbeck</t>
+  </si>
+  <si>
+    <t>Netz</t>
+  </si>
+  <si>
+    <t>Tschernuth</t>
+  </si>
+  <si>
+    <t>Petersson</t>
+  </si>
+  <si>
+    <t>M. El Mala</t>
+  </si>
+  <si>
+    <t>14.06.2025</t>
+  </si>
 </sst>
 </file>
 
@@ -1348,7 +1369,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{93EB6F54-7766-4759-97DF-03549A275A7C}">
-  <dimension ref="A1:M1135"/>
+  <dimension ref="A1:M1220"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.90625" style="2"/>
@@ -44049,7 +44070,3272 @@
       </c>
     </row>
     <row r="1135" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="M1135" s="7"/>
+      <c r="B1135" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1135" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1135" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1135" s="2">
+        <v>70</v>
+      </c>
+      <c r="F1135" s="3">
+        <v>1770000</v>
+      </c>
+      <c r="G1135" s="3">
+        <v>1780000</v>
+      </c>
+      <c r="H1135" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="I1135" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1135" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1135" s="2">
+        <v>1</v>
+      </c>
+      <c r="L1135" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="M1135" s="7" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="1136" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B1136" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="C1136" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1136" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="E1136" s="2">
+        <v>124</v>
+      </c>
+      <c r="F1136" s="3">
+        <v>5570000</v>
+      </c>
+      <c r="G1136" s="3">
+        <v>5400000</v>
+      </c>
+      <c r="H1136" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="I1136" s="2" t="s">
+        <v>274</v>
+      </c>
+      <c r="J1136" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1136" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1136" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="M1136" s="7" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="1137" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1137" s="2" t="s">
+        <v>281</v>
+      </c>
+      <c r="C1137" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1137" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="E1137" s="2">
+        <v>143</v>
+      </c>
+      <c r="F1137" s="3">
+        <v>5690000</v>
+      </c>
+      <c r="G1137" s="3">
+        <v>5530000</v>
+      </c>
+      <c r="H1137" s="2" t="s">
+        <v>282</v>
+      </c>
+      <c r="I1137" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1137" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1137" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1137" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="M1137" s="7" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="1138" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1138" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="C1138" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1138" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E1138" s="2">
+        <v>128</v>
+      </c>
+      <c r="F1138" s="3">
+        <v>4610000</v>
+      </c>
+      <c r="G1138" s="3">
+        <v>4540000</v>
+      </c>
+      <c r="H1138" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="I1138" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1138" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1138" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1138" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="M1138" s="7" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="1139" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1139" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="C1139" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1139" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="E1139" s="2">
+        <v>83</v>
+      </c>
+      <c r="F1139" s="3">
+        <v>950000</v>
+      </c>
+      <c r="G1139" s="3">
+        <v>980000</v>
+      </c>
+      <c r="H1139" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="I1139" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1139" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1139" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1139" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="M1139" s="7" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="1140" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1140" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1140" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1140" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E1140" s="2">
+        <v>43</v>
+      </c>
+      <c r="F1140" s="3">
+        <v>2370000</v>
+      </c>
+      <c r="G1140" s="3">
+        <v>2400000</v>
+      </c>
+      <c r="H1140" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="I1140" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1140" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1140" s="2">
+        <v>1</v>
+      </c>
+      <c r="L1140" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="M1140" s="7" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="1141" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1141" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1141" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1141" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E1141" s="2">
+        <v>42</v>
+      </c>
+      <c r="F1141" s="3">
+        <v>5230000</v>
+      </c>
+      <c r="G1141" s="3">
+        <v>5170000</v>
+      </c>
+      <c r="H1141" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="I1141" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1141" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1141" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1141" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="M1141" s="7" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="1142" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1142" s="2" t="s">
+        <v>220</v>
+      </c>
+      <c r="C1142" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1142" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="E1142" s="2">
+        <v>43</v>
+      </c>
+      <c r="F1142" s="3">
+        <v>4190000</v>
+      </c>
+      <c r="G1142" s="3">
+        <v>4170000</v>
+      </c>
+      <c r="H1142" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="I1142" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1142" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="K1142" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1142" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="M1142" s="7" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="1143" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1143" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="C1143" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1143" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="E1143" s="2">
+        <v>60</v>
+      </c>
+      <c r="F1143" s="3">
+        <v>1250000</v>
+      </c>
+      <c r="G1143" s="3">
+        <v>1250000</v>
+      </c>
+      <c r="H1143" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="I1143" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1143" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1143" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1143" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="M1143" s="7" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="1144" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1144" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C1144" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1144" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="E1144" s="2">
+        <v>124</v>
+      </c>
+      <c r="F1144" s="3">
+        <v>3310000</v>
+      </c>
+      <c r="G1144" s="3">
+        <v>3290000</v>
+      </c>
+      <c r="H1144" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="I1144" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1144" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1144" s="2">
+        <v>1</v>
+      </c>
+      <c r="L1144" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="M1144" s="7" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="1145" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1145" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1145" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1145" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E1145" s="2">
+        <v>112</v>
+      </c>
+      <c r="F1145" s="3">
+        <v>4390000</v>
+      </c>
+      <c r="G1145" s="3">
+        <v>4370000</v>
+      </c>
+      <c r="H1145" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="I1145" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1145" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1145" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1145" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="M1145" s="7" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="1146" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1146" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="C1146" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1146" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="E1146" s="2">
+        <v>108</v>
+      </c>
+      <c r="F1146" s="3">
+        <v>3850000</v>
+      </c>
+      <c r="G1146" s="3">
+        <v>3790000</v>
+      </c>
+      <c r="H1146" s="2" t="s">
+        <v>264</v>
+      </c>
+      <c r="I1146" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1146" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1146" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1146" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="M1146" s="7" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="1147" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1147" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="C1147" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1147" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="E1147" s="2">
+        <v>183</v>
+      </c>
+      <c r="F1147" s="3">
+        <v>9970000</v>
+      </c>
+      <c r="G1147" s="3">
+        <v>9880000</v>
+      </c>
+      <c r="H1147" s="2" t="s">
+        <v>236</v>
+      </c>
+      <c r="I1147" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1147" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="K1147" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1147" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="M1147" s="7" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="1148" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1148" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="C1148" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1148" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E1148" s="2">
+        <v>167</v>
+      </c>
+      <c r="F1148" s="3">
+        <v>9150000</v>
+      </c>
+      <c r="G1148" s="3">
+        <v>9100000</v>
+      </c>
+      <c r="H1148" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="I1148" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1148" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1148" s="2">
+        <v>1</v>
+      </c>
+      <c r="L1148" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="M1148" s="7" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="1149" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1149" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C1149" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1149" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="E1149" s="2">
+        <v>127</v>
+      </c>
+      <c r="F1149" s="3">
+        <v>3000000</v>
+      </c>
+      <c r="G1149" s="3">
+        <v>3030000</v>
+      </c>
+      <c r="H1149" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="I1149" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1149" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1149" s="2">
+        <v>1</v>
+      </c>
+      <c r="L1149" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="M1149" s="7" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="1150" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1150" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="C1150" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1150" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E1150" s="2">
+        <v>69</v>
+      </c>
+      <c r="F1150" s="3">
+        <v>1750000</v>
+      </c>
+      <c r="G1150" s="3">
+        <v>1770000</v>
+      </c>
+      <c r="H1150" s="2" t="s">
+        <v>241</v>
+      </c>
+      <c r="I1150" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1150" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1150" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1150" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="M1150" s="7" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="1151" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1151" s="2" t="s">
+        <v>295</v>
+      </c>
+      <c r="C1151" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1151" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="E1151" s="2">
+        <v>100</v>
+      </c>
+      <c r="F1151" s="3">
+        <v>2540000</v>
+      </c>
+      <c r="G1151" s="3">
+        <v>2480000</v>
+      </c>
+      <c r="H1151" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="I1151" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1151" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1151" s="2">
+        <v>2</v>
+      </c>
+      <c r="L1151" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1151" s="7" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="1152" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1152" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C1152" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1152" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="E1152" s="2">
+        <v>72</v>
+      </c>
+      <c r="F1152" s="3">
+        <v>1820000</v>
+      </c>
+      <c r="G1152" s="3">
+        <v>1810000</v>
+      </c>
+      <c r="H1152" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="I1152" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1152" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1152" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1152" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="M1152" s="7" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="1153" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1153" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="C1153" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1153" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="E1153" s="2">
+        <v>0</v>
+      </c>
+      <c r="F1153" s="3">
+        <v>2580000</v>
+      </c>
+      <c r="G1153" s="3">
+        <v>2590000</v>
+      </c>
+      <c r="H1153" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="I1153" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1153" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1153" s="2">
+        <v>1</v>
+      </c>
+      <c r="L1153" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="M1153" s="7" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="1154" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1154" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="C1154" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1154" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="E1154" s="2">
+        <v>0</v>
+      </c>
+      <c r="F1154" s="3">
+        <v>2150000</v>
+      </c>
+      <c r="G1154" s="3">
+        <v>2170000</v>
+      </c>
+      <c r="H1154" s="2" t="s">
+        <v>244</v>
+      </c>
+      <c r="I1154" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1154" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="K1154" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1154" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="M1154" s="7" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="1155" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1155" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C1155" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1155" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="E1155" s="2">
+        <v>110</v>
+      </c>
+      <c r="F1155" s="3">
+        <v>3420000</v>
+      </c>
+      <c r="G1155" s="3">
+        <v>3410000</v>
+      </c>
+      <c r="H1155" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="I1155" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1155" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1155" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1155" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="M1155" s="7" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="1156" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1156" s="2" t="s">
+        <v>284</v>
+      </c>
+      <c r="C1156" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1156" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1156" s="2">
+        <v>0</v>
+      </c>
+      <c r="F1156" s="3">
+        <v>3610000</v>
+      </c>
+      <c r="G1156" s="3">
+        <v>3600000</v>
+      </c>
+      <c r="H1156" s="2" t="s">
+        <v>285</v>
+      </c>
+      <c r="I1156" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1156" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1156" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1156" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="M1156" s="7" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="1157" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1157" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C1157" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1157" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1157" s="2">
+        <v>0</v>
+      </c>
+      <c r="F1157" s="3">
+        <v>3110000</v>
+      </c>
+      <c r="G1157" s="3">
+        <v>3100000</v>
+      </c>
+      <c r="H1157" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="I1157" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1157" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1157" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1157" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="M1157" s="7" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="1158" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1158" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="C1158" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1158" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="E1158" s="2">
+        <v>95</v>
+      </c>
+      <c r="F1158" s="3">
+        <v>3560000</v>
+      </c>
+      <c r="G1158" s="3">
+        <v>3580000</v>
+      </c>
+      <c r="H1158" s="2" t="s">
+        <v>285</v>
+      </c>
+      <c r="I1158" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1158" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1158" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1158" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="M1158" s="7" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="1159" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1159" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="C1159" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1159" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="E1159" s="2">
+        <v>71</v>
+      </c>
+      <c r="F1159" s="3">
+        <v>1440000</v>
+      </c>
+      <c r="G1159" s="3">
+        <v>1440000</v>
+      </c>
+      <c r="H1159" s="2" t="s">
+        <v>238</v>
+      </c>
+      <c r="I1159" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1159" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1159" s="2">
+        <v>1</v>
+      </c>
+      <c r="L1159" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="M1159" s="7" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="1160" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1160" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C1160" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1160" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="E1160" s="2">
+        <v>127</v>
+      </c>
+      <c r="F1160" s="3">
+        <v>5380000</v>
+      </c>
+      <c r="G1160" s="3">
+        <v>5350000</v>
+      </c>
+      <c r="H1160" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="I1160" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1160" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1160" s="2">
+        <v>1</v>
+      </c>
+      <c r="L1160" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="M1160" s="7" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="1161" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1161" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C1161" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1161" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="E1161" s="2">
+        <v>8</v>
+      </c>
+      <c r="F1161" s="3">
+        <v>230000</v>
+      </c>
+      <c r="G1161" s="3">
+        <v>230000</v>
+      </c>
+      <c r="H1161" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="I1161" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1161" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1161" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1161" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="M1161" s="7" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="1162" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1162" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C1162" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1162" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="E1162" s="2">
+        <v>72</v>
+      </c>
+      <c r="F1162" s="3">
+        <v>3070000</v>
+      </c>
+      <c r="G1162" s="3">
+        <v>3070000</v>
+      </c>
+      <c r="H1162" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="I1162" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1162" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1162" s="2">
+        <v>1</v>
+      </c>
+      <c r="L1162" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="M1162" s="7" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="1163" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1163" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="C1163" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1163" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="E1163" s="2">
+        <v>36</v>
+      </c>
+      <c r="F1163" s="3">
+        <v>3020000</v>
+      </c>
+      <c r="G1163" s="3">
+        <v>3060000</v>
+      </c>
+      <c r="H1163" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="I1163" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1163" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="K1163" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1163" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="M1163" s="7" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="1164" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1164" s="2" t="s">
+        <v>286</v>
+      </c>
+      <c r="C1164" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1164" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="E1164" s="2">
+        <v>184</v>
+      </c>
+      <c r="F1164" s="3">
+        <v>15550000</v>
+      </c>
+      <c r="G1164" s="3">
+        <v>15660000</v>
+      </c>
+      <c r="H1164" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="I1164" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1164" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1164" s="2">
+        <v>2</v>
+      </c>
+      <c r="L1164" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1164" s="7" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="1165" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1165" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="C1165" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1165" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="E1165" s="2">
+        <v>87</v>
+      </c>
+      <c r="F1165" s="3">
+        <v>2550000</v>
+      </c>
+      <c r="G1165" s="3">
+        <v>2540000</v>
+      </c>
+      <c r="H1165" s="2" t="s">
+        <v>238</v>
+      </c>
+      <c r="I1165" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1165" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1165" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1165" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="M1165" s="7" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="1166" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1166" s="2" t="s">
+        <v>296</v>
+      </c>
+      <c r="C1166" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1166" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="E1166" s="2">
+        <v>95</v>
+      </c>
+      <c r="F1166" s="3">
+        <v>6890000</v>
+      </c>
+      <c r="G1166" s="3">
+        <v>6960000</v>
+      </c>
+      <c r="H1166" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="I1166" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="J1166" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="K1166" s="2">
+        <v>2</v>
+      </c>
+      <c r="L1166" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1166" s="7" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="1167" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1167" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="C1167" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1167" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="E1167" s="2">
+        <v>123</v>
+      </c>
+      <c r="F1167" s="3">
+        <v>3560000</v>
+      </c>
+      <c r="G1167" s="3">
+        <v>3630000</v>
+      </c>
+      <c r="H1167" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="I1167" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1167" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1167" s="2">
+        <v>1</v>
+      </c>
+      <c r="L1167" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="M1167" s="7" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="1168" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1168" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="C1168" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1168" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="E1168" s="2">
+        <v>89</v>
+      </c>
+      <c r="F1168" s="3">
+        <v>1750000</v>
+      </c>
+      <c r="G1168" s="3">
+        <v>1770000</v>
+      </c>
+      <c r="H1168" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="I1168" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1168" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1168" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1168" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="M1168" s="7" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="1169" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1169" s="2" t="s">
+        <v>288</v>
+      </c>
+      <c r="C1169" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1169" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="E1169" s="2">
+        <v>0</v>
+      </c>
+      <c r="F1169" s="3">
+        <v>210000</v>
+      </c>
+      <c r="G1169" s="3">
+        <v>210000</v>
+      </c>
+      <c r="H1169" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="I1169" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1169" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="K1169" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1169" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1169" s="7" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="1170" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1170" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="C1170" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1170" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E1170" s="2">
+        <v>77</v>
+      </c>
+      <c r="F1170" s="3">
+        <v>2200000</v>
+      </c>
+      <c r="G1170" s="3">
+        <v>2210000</v>
+      </c>
+      <c r="H1170" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="I1170" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1170" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1170" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1170" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="M1170" s="7" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="1171" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1171" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="C1171" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1171" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E1171" s="2">
+        <v>100</v>
+      </c>
+      <c r="F1171" s="3">
+        <v>4650000</v>
+      </c>
+      <c r="G1171" s="3">
+        <v>4690000</v>
+      </c>
+      <c r="H1171" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="I1171" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1171" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1171" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1171" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="M1171" s="7" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="1172" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1172" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="C1172" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1172" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1172" s="2">
+        <v>199</v>
+      </c>
+      <c r="F1172" s="3">
+        <v>18620000</v>
+      </c>
+      <c r="G1172" s="3">
+        <v>18700000</v>
+      </c>
+      <c r="H1172" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="I1172" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1172" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1172" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1172" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="M1172" s="7" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="1173" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1173" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="C1173" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1173" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="E1173" s="2">
+        <v>179</v>
+      </c>
+      <c r="F1173" s="3">
+        <v>11630000</v>
+      </c>
+      <c r="G1173" s="3">
+        <v>11600000</v>
+      </c>
+      <c r="H1173" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="I1173" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1173" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1173" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1173" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="M1173" s="7" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="1174" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1174" s="2" t="s">
+        <v>276</v>
+      </c>
+      <c r="C1174" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1174" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E1174" s="2">
+        <v>7</v>
+      </c>
+      <c r="F1174" s="3">
+        <v>320000</v>
+      </c>
+      <c r="G1174" s="3">
+        <v>320000</v>
+      </c>
+      <c r="H1174" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="I1174" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1174" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1174" s="2">
+        <v>1</v>
+      </c>
+      <c r="L1174" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1174" s="7" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="1175" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1175" s="2" t="s">
+        <v>297</v>
+      </c>
+      <c r="C1175" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1175" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="E1175" s="2">
+        <v>46</v>
+      </c>
+      <c r="F1175" s="3">
+        <v>1320000</v>
+      </c>
+      <c r="G1175" s="3">
+        <v>1330000</v>
+      </c>
+      <c r="H1175" s="2" t="s">
+        <v>271</v>
+      </c>
+      <c r="I1175" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1175" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1175" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1175" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1175" s="7" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="1176" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1176" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="C1176" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1176" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E1176" s="2">
+        <v>185</v>
+      </c>
+      <c r="F1176" s="3">
+        <v>12160000</v>
+      </c>
+      <c r="G1176" s="3">
+        <v>12220000</v>
+      </c>
+      <c r="H1176" s="2" t="s">
+        <v>255</v>
+      </c>
+      <c r="I1176" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1176" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1176" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1176" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="M1176" s="7" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="1177" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1177" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="C1177" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1177" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1177" s="2">
+        <v>0</v>
+      </c>
+      <c r="F1177" s="3">
+        <v>4060000</v>
+      </c>
+      <c r="G1177" s="3">
+        <v>4050000</v>
+      </c>
+      <c r="H1177" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="I1177" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1177" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1177" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1177" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="M1177" s="7" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="1178" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1178" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="C1178" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1178" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E1178" s="2">
+        <v>51</v>
+      </c>
+      <c r="F1178" s="3">
+        <v>2570000</v>
+      </c>
+      <c r="G1178" s="3">
+        <v>2630000</v>
+      </c>
+      <c r="H1178" s="2" t="s">
+        <v>246</v>
+      </c>
+      <c r="I1178" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1178" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1178" s="2">
+        <v>1</v>
+      </c>
+      <c r="L1178" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="M1178" s="7" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="1179" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1179" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="C1179" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1179" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E1179" s="2">
+        <v>119</v>
+      </c>
+      <c r="F1179" s="3">
+        <v>5930000</v>
+      </c>
+      <c r="G1179" s="3">
+        <v>5940000</v>
+      </c>
+      <c r="H1179" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="I1179" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1179" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1179" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1179" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="M1179" s="7" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="1180" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1180" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="C1180" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1180" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E1180" s="2">
+        <v>127</v>
+      </c>
+      <c r="F1180" s="3">
+        <v>6290000</v>
+      </c>
+      <c r="G1180" s="3">
+        <v>6170000</v>
+      </c>
+      <c r="H1180" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="I1180" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1180" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1180" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1180" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="M1180" s="7" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="1181" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1181" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="C1181" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1181" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E1181" s="2">
+        <v>69</v>
+      </c>
+      <c r="F1181" s="3">
+        <v>4700000</v>
+      </c>
+      <c r="G1181" s="3">
+        <v>4770000</v>
+      </c>
+      <c r="H1181" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="I1181" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1181" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1181" s="2">
+        <v>1</v>
+      </c>
+      <c r="L1181" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="M1181" s="7" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="1182" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1182" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="C1182" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1182" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1182" s="2">
+        <v>68</v>
+      </c>
+      <c r="F1182" s="3">
+        <v>4220000</v>
+      </c>
+      <c r="G1182" s="3">
+        <v>4250000</v>
+      </c>
+      <c r="H1182" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="I1182" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1182" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="K1182" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1182" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="M1182" s="7" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="1183" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1183" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="C1183" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1183" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="E1183" s="2">
+        <v>81</v>
+      </c>
+      <c r="F1183" s="3">
+        <v>1520000</v>
+      </c>
+      <c r="G1183" s="3">
+        <v>1510000</v>
+      </c>
+      <c r="H1183" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="I1183" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1183" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1183" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1183" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="M1183" s="7" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="1184" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1184" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="C1184" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1184" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="E1184" s="2">
+        <v>123</v>
+      </c>
+      <c r="F1184" s="3">
+        <v>5020000</v>
+      </c>
+      <c r="G1184" s="3">
+        <v>4990000</v>
+      </c>
+      <c r="H1184" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="I1184" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1184" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1184" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1184" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="M1184" s="7" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="1185" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1185" s="2" t="s">
+        <v>289</v>
+      </c>
+      <c r="C1185" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1185" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="E1185" s="2">
+        <v>128</v>
+      </c>
+      <c r="F1185" s="3">
+        <v>4720000</v>
+      </c>
+      <c r="G1185" s="3">
+        <v>4680000</v>
+      </c>
+      <c r="H1185" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="I1185" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1185" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1185" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1185" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="M1185" s="7" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="1186" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1186" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="C1186" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1186" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="E1186" s="2">
+        <v>109</v>
+      </c>
+      <c r="F1186" s="3">
+        <v>3540000</v>
+      </c>
+      <c r="G1186" s="3">
+        <v>3580000</v>
+      </c>
+      <c r="H1186" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="I1186" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1186" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1186" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1186" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="M1186" s="7" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="1187" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1187" s="2" t="s">
+        <v>290</v>
+      </c>
+      <c r="C1187" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1187" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1187" s="2">
+        <v>0</v>
+      </c>
+      <c r="F1187" s="3">
+        <v>160000</v>
+      </c>
+      <c r="G1187" s="3">
+        <v>160000</v>
+      </c>
+      <c r="H1187" s="2" t="s">
+        <v>291</v>
+      </c>
+      <c r="I1187" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1187" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="K1187" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1187" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1187" s="7" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="1188" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1188" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="C1188" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1188" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E1188" s="2">
+        <v>0</v>
+      </c>
+      <c r="F1188" s="3">
+        <v>1940000</v>
+      </c>
+      <c r="G1188" s="3">
+        <v>1940000</v>
+      </c>
+      <c r="H1188" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="I1188" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1188" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="K1188" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1188" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="M1188" s="7" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="1189" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1189" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="C1189" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1189" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="E1189" s="2">
+        <v>12</v>
+      </c>
+      <c r="F1189" s="3">
+        <v>710000</v>
+      </c>
+      <c r="G1189" s="3">
+        <v>690000</v>
+      </c>
+      <c r="H1189" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="I1189" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1189" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1189" s="2">
+        <v>1</v>
+      </c>
+      <c r="L1189" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="M1189" s="7" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="1190" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1190" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="C1190" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1190" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E1190" s="2">
+        <v>0</v>
+      </c>
+      <c r="F1190" s="3">
+        <v>9870000</v>
+      </c>
+      <c r="G1190" s="3">
+        <v>10270000</v>
+      </c>
+      <c r="H1190" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="I1190" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1190" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="K1190" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1190" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="M1190" s="7" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="1191" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1191" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="C1191" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1191" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E1191" s="2">
+        <v>118</v>
+      </c>
+      <c r="F1191" s="3">
+        <v>6350000</v>
+      </c>
+      <c r="G1191" s="3">
+        <v>6230000</v>
+      </c>
+      <c r="H1191" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="I1191" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1191" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1191" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1191" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="M1191" s="7" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="1192" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1192" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="C1192" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1192" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E1192" s="2">
+        <v>30</v>
+      </c>
+      <c r="F1192" s="3">
+        <v>2480000</v>
+      </c>
+      <c r="G1192" s="3">
+        <v>2620000</v>
+      </c>
+      <c r="H1192" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="I1192" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1192" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1192" s="2">
+        <v>5</v>
+      </c>
+      <c r="L1192" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1192" s="7" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="1193" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1193" s="2" t="s">
+        <v>298</v>
+      </c>
+      <c r="C1193" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1193" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="E1193" s="2">
+        <v>0</v>
+      </c>
+      <c r="F1193" s="3">
+        <v>160000</v>
+      </c>
+      <c r="G1193" s="3">
+        <v>160000</v>
+      </c>
+      <c r="H1193" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="I1193" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1193" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="K1193" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1193" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1193" s="7" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="1194" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1194" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="C1194" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1194" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E1194" s="2">
+        <v>54</v>
+      </c>
+      <c r="F1194" s="3">
+        <v>2300000</v>
+      </c>
+      <c r="G1194" s="3">
+        <v>2290000</v>
+      </c>
+      <c r="H1194" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="I1194" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1194" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1194" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1194" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="M1194" s="7" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="1195" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1195" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="C1195" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1195" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E1195" s="2">
+        <v>89</v>
+      </c>
+      <c r="F1195" s="3">
+        <v>8240000</v>
+      </c>
+      <c r="G1195" s="3">
+        <v>8240000</v>
+      </c>
+      <c r="H1195" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="I1195" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1195" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1195" s="2">
+        <v>1</v>
+      </c>
+      <c r="L1195" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="M1195" s="7" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="1196" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1196" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="C1196" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1196" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="E1196" s="2">
+        <v>130</v>
+      </c>
+      <c r="F1196" s="3">
+        <v>11820000</v>
+      </c>
+      <c r="G1196" s="3">
+        <v>11950000</v>
+      </c>
+      <c r="H1196" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="I1196" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1196" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1196" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1196" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="M1196" s="7" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="1197" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1197" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="C1197" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1197" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1197" s="2">
+        <v>0</v>
+      </c>
+      <c r="F1197" s="3">
+        <v>1890000</v>
+      </c>
+      <c r="G1197" s="3">
+        <v>1880000</v>
+      </c>
+      <c r="H1197" s="2" t="s">
+        <v>241</v>
+      </c>
+      <c r="I1197" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1197" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1197" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1197" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="M1197" s="7" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="1198" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1198" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="C1198" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1198" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="E1198" s="2">
+        <v>41</v>
+      </c>
+      <c r="F1198" s="3">
+        <v>1110000</v>
+      </c>
+      <c r="G1198" s="3">
+        <v>1090000</v>
+      </c>
+      <c r="H1198" s="2" t="s">
+        <v>285</v>
+      </c>
+      <c r="I1198" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1198" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1198" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1198" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="M1198" s="7" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="1199" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1199" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="C1199" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1199" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1199" s="2">
+        <v>91</v>
+      </c>
+      <c r="F1199" s="3">
+        <v>7920000</v>
+      </c>
+      <c r="G1199" s="3">
+        <v>7980000</v>
+      </c>
+      <c r="H1199" s="2" t="s">
+        <v>264</v>
+      </c>
+      <c r="I1199" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1199" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1199" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1199" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="M1199" s="7" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="1200" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1200" s="2" t="s">
+        <v>292</v>
+      </c>
+      <c r="C1200" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1200" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="E1200" s="2">
+        <v>30</v>
+      </c>
+      <c r="F1200" s="3">
+        <v>870000</v>
+      </c>
+      <c r="G1200" s="3">
+        <v>860000</v>
+      </c>
+      <c r="H1200" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="I1200" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1200" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1200" s="2">
+        <v>1</v>
+      </c>
+      <c r="L1200" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1200" s="7" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="1201" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1201" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="C1201" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1201" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="E1201" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1201" s="3">
+        <v>270000</v>
+      </c>
+      <c r="G1201" s="3">
+        <v>270000</v>
+      </c>
+      <c r="H1201" s="2" t="s">
+        <v>244</v>
+      </c>
+      <c r="I1201" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1201" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="K1201" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1201" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="M1201" s="7" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="1202" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1202" s="2" t="s">
+        <v>299</v>
+      </c>
+      <c r="C1202" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1202" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E1202" s="2">
+        <v>0</v>
+      </c>
+      <c r="F1202" s="3">
+        <v>160000</v>
+      </c>
+      <c r="G1202" s="3">
+        <v>160000</v>
+      </c>
+      <c r="H1202" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="I1202" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1202" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="K1202" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1202" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1202" s="7" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="1203" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1203" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="C1203" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1203" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="E1203" s="2">
+        <v>108</v>
+      </c>
+      <c r="F1203" s="3">
+        <v>3210000</v>
+      </c>
+      <c r="G1203" s="3">
+        <v>3160000</v>
+      </c>
+      <c r="H1203" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="I1203" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1203" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1203" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1203" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="M1203" s="7" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="1204" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1204" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="C1204" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1204" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="E1204" s="2">
+        <v>112</v>
+      </c>
+      <c r="F1204" s="3">
+        <v>4070000</v>
+      </c>
+      <c r="G1204" s="3">
+        <v>4030000</v>
+      </c>
+      <c r="H1204" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="I1204" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="J1204" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1204" s="2">
+        <v>1</v>
+      </c>
+      <c r="L1204" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="M1204" s="7" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="1205" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1205" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="C1205" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1205" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="E1205" s="2">
+        <v>90</v>
+      </c>
+      <c r="F1205" s="3">
+        <v>3580000</v>
+      </c>
+      <c r="G1205" s="3">
+        <v>3590000</v>
+      </c>
+      <c r="H1205" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="I1205" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1205" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1205" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1205" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="M1205" s="7" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="1206" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1206" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="C1206" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1206" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="E1206" s="2">
+        <v>15</v>
+      </c>
+      <c r="F1206" s="3">
+        <v>370000</v>
+      </c>
+      <c r="G1206" s="3">
+        <v>380000</v>
+      </c>
+      <c r="H1206" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="I1206" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1206" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1206" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1206" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="M1206" s="7" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="1207" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1207" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="C1207" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1207" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="E1207" s="2">
+        <v>58</v>
+      </c>
+      <c r="F1207" s="3">
+        <v>1210000</v>
+      </c>
+      <c r="G1207" s="3">
+        <v>1220000</v>
+      </c>
+      <c r="H1207" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="I1207" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1207" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1207" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1207" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="M1207" s="7" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="1208" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1208" s="2" t="s">
+        <v>293</v>
+      </c>
+      <c r="C1208" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1208" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="E1208" s="2">
+        <v>48</v>
+      </c>
+      <c r="F1208" s="3">
+        <v>1530000</v>
+      </c>
+      <c r="G1208" s="3">
+        <v>1540000</v>
+      </c>
+      <c r="H1208" s="2" t="s">
+        <v>246</v>
+      </c>
+      <c r="I1208" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1208" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1208" s="2">
+        <v>5</v>
+      </c>
+      <c r="L1208" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1208" s="7" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="1209" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1209" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="C1209" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1209" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E1209" s="2">
+        <v>77</v>
+      </c>
+      <c r="F1209" s="3">
+        <v>4310000</v>
+      </c>
+      <c r="G1209" s="3">
+        <v>4360000</v>
+      </c>
+      <c r="H1209" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="I1209" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1209" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1209" s="2">
+        <v>1</v>
+      </c>
+      <c r="L1209" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="M1209" s="7" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="1210" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1210" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="C1210" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1210" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="E1210" s="2">
+        <v>4</v>
+      </c>
+      <c r="F1210" s="3">
+        <v>390000</v>
+      </c>
+      <c r="G1210" s="3">
+        <v>390000</v>
+      </c>
+      <c r="H1210" s="2" t="s">
+        <v>244</v>
+      </c>
+      <c r="I1210" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1210" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="K1210" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1210" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="M1210" s="7" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="1211" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1211" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="C1211" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1211" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E1211" s="2">
+        <v>47</v>
+      </c>
+      <c r="F1211" s="3">
+        <v>1290000</v>
+      </c>
+      <c r="G1211" s="3">
+        <v>1290000</v>
+      </c>
+      <c r="H1211" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="I1211" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1211" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1211" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1211" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="M1211" s="7" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="1212" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1212" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="C1212" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1212" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E1212" s="2">
+        <v>156</v>
+      </c>
+      <c r="F1212" s="3">
+        <v>6470000</v>
+      </c>
+      <c r="G1212" s="3">
+        <v>6350000</v>
+      </c>
+      <c r="H1212" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="I1212" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1212" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1212" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1212" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="M1212" s="7" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="1213" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1213" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="C1213" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1213" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="E1213" s="2">
+        <v>29</v>
+      </c>
+      <c r="F1213" s="3">
+        <v>790000</v>
+      </c>
+      <c r="G1213" s="3">
+        <v>800000</v>
+      </c>
+      <c r="H1213" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="I1213" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1213" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1213" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1213" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="M1213" s="7" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="1214" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1214" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="C1214" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1214" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E1214" s="2">
+        <v>102</v>
+      </c>
+      <c r="F1214" s="3">
+        <v>2990000</v>
+      </c>
+      <c r="G1214" s="3">
+        <v>2940000</v>
+      </c>
+      <c r="H1214" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="I1214" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1214" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1214" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1214" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="M1214" s="7" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="1215" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1215" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="C1215" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1215" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E1215" s="2">
+        <v>11</v>
+      </c>
+      <c r="F1215" s="3">
+        <v>2870000</v>
+      </c>
+      <c r="G1215" s="3">
+        <v>2850000</v>
+      </c>
+      <c r="H1215" s="2" t="s">
+        <v>265</v>
+      </c>
+      <c r="I1215" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1215" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="K1215" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1215" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="M1215" s="7" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="1216" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1216" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="C1216" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1216" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="E1216" s="2">
+        <v>17</v>
+      </c>
+      <c r="F1216" s="3">
+        <v>1350000</v>
+      </c>
+      <c r="G1216" s="3">
+        <v>1350000</v>
+      </c>
+      <c r="H1216" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="I1216" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1216" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1216" s="2">
+        <v>1</v>
+      </c>
+      <c r="L1216" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="M1216" s="7" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="1217" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1217" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="C1217" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1217" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="E1217" s="2">
+        <v>0</v>
+      </c>
+      <c r="F1217" s="3">
+        <v>160000</v>
+      </c>
+      <c r="G1217" s="3">
+        <v>160000</v>
+      </c>
+      <c r="H1217" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="I1217" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1217" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="K1217" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1217" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1217" s="7" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="1218" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1218" s="2" t="s">
+        <v>300</v>
+      </c>
+      <c r="C1218" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1218" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1218" s="2">
+        <v>0</v>
+      </c>
+      <c r="F1218" s="3">
+        <v>420000</v>
+      </c>
+      <c r="G1218" s="3">
+        <v>430000</v>
+      </c>
+      <c r="H1218" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="I1218" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1218" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="K1218" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1218" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1218" s="7" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="1219" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1219" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="C1219" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1219" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="E1219" s="2">
+        <v>0</v>
+      </c>
+      <c r="F1219" s="3">
+        <v>3450000</v>
+      </c>
+      <c r="G1219" s="3">
+        <v>3410000</v>
+      </c>
+      <c r="H1219" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="I1219" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1219" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="K1219" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1219" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="M1219" s="7" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="1220" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1220" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="C1220" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1220" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="E1220" s="2">
+        <v>0</v>
+      </c>
+      <c r="F1220" s="3">
+        <v>180000</v>
+      </c>
+      <c r="G1220" s="3">
+        <v>180000</v>
+      </c>
+      <c r="H1220" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="I1220" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1220" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="K1220" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1220" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1220" s="7" t="s">
+        <v>301</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="B1:M1" xr:uid="{93EB6F54-7766-4759-97DF-03549A275A7C}">

</xml_diff>

<commit_message>
Automatisches Update TM + Transfers - 15.06.2025 16:41
</commit_message>
<xml_diff>
--- a/TM_all.xlsx
+++ b/TM_all.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/aecf56309e6168f4/Documents/comunio/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="239" documentId="8_{B00F7E9F-5C85-449B-834E-0179FBCEE2D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E2CB34A4-E516-4A1A-8BA5-8CA4166C45EF}"/>
+  <xr:revisionPtr revIDLastSave="244" documentId="8_{B00F7E9F-5C85-449B-834E-0179FBCEE2D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6E3F379B-9358-4168-BFDA-3998CC4AE001}"/>
   <bookViews>
-    <workbookView xWindow="6660" yWindow="2700" windowWidth="28800" windowHeight="15370" xr2:uid="{607DE709-F91E-4262-9941-1066BBEC319E}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{607DE709-F91E-4262-9941-1066BBEC319E}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8675" uniqueCount="302">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9443" uniqueCount="309">
   <si>
     <t>Spieler</t>
   </si>
@@ -946,6 +946,27 @@
   <si>
     <t>14.06.2025</t>
   </si>
+  <si>
+    <t>Heintz</t>
+  </si>
+  <si>
+    <t>Ritzka</t>
+  </si>
+  <si>
+    <t>Kaufmann</t>
+  </si>
+  <si>
+    <t>Kim</t>
+  </si>
+  <si>
+    <t>Heitmann</t>
+  </si>
+  <si>
+    <t>Telle</t>
+  </si>
+  <si>
+    <t>15.06.2025</t>
+  </si>
 </sst>
 </file>
 
@@ -1369,7 +1390,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{93EB6F54-7766-4759-97DF-03549A275A7C}">
-  <dimension ref="A1:M1220"/>
+  <dimension ref="A1:M1316"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.90625" style="2"/>
@@ -47335,6 +47356,3654 @@
       </c>
       <c r="M1220" s="7" t="s">
         <v>301</v>
+      </c>
+    </row>
+    <row r="1221" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1221" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1221" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1221" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1221" s="2">
+        <v>70</v>
+      </c>
+      <c r="F1221" s="3">
+        <v>1980000</v>
+      </c>
+      <c r="G1221" s="3">
+        <v>1960000</v>
+      </c>
+      <c r="H1221" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="I1221" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1221" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1221" s="2">
+        <v>1</v>
+      </c>
+      <c r="L1221" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="M1221" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1222" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1222" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="C1222" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1222" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="E1222" s="2">
+        <v>124</v>
+      </c>
+      <c r="F1222" s="3">
+        <v>5600000</v>
+      </c>
+      <c r="G1222" s="3">
+        <v>5480000</v>
+      </c>
+      <c r="H1222" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="I1222" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1222" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1222" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1222" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="M1222" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1223" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1223" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1223" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1223" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E1223" s="2">
+        <v>95</v>
+      </c>
+      <c r="F1223" s="3">
+        <v>3780000</v>
+      </c>
+      <c r="G1223" s="3">
+        <v>3930000</v>
+      </c>
+      <c r="H1223" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="I1223" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1223" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1223" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1223" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="M1223" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1224" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1224" s="2" t="s">
+        <v>281</v>
+      </c>
+      <c r="C1224" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1224" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="E1224" s="2">
+        <v>143</v>
+      </c>
+      <c r="F1224" s="3">
+        <v>5610000</v>
+      </c>
+      <c r="G1224" s="3">
+        <v>5430000</v>
+      </c>
+      <c r="H1224" s="2" t="s">
+        <v>282</v>
+      </c>
+      <c r="I1224" s="2" t="s">
+        <v>274</v>
+      </c>
+      <c r="J1224" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1224" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1224" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="M1224" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1225" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1225" s="2" t="s">
+        <v>302</v>
+      </c>
+      <c r="C1225" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1225" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1225" s="2">
+        <v>0</v>
+      </c>
+      <c r="F1225" s="3">
+        <v>1670000</v>
+      </c>
+      <c r="G1225" s="3">
+        <v>1660000</v>
+      </c>
+      <c r="H1225" s="2" t="s">
+        <v>247</v>
+      </c>
+      <c r="I1225" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1225" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1225" s="2">
+        <v>1</v>
+      </c>
+      <c r="L1225" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1225" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1226" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1226" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="C1226" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1226" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E1226" s="2">
+        <v>128</v>
+      </c>
+      <c r="F1226" s="3">
+        <v>4670000</v>
+      </c>
+      <c r="G1226" s="3">
+        <v>4680000</v>
+      </c>
+      <c r="H1226" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="I1226" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1226" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1226" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1226" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="M1226" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1227" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1227" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="C1227" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1227" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="E1227" s="2">
+        <v>83</v>
+      </c>
+      <c r="F1227" s="3">
+        <v>980000</v>
+      </c>
+      <c r="G1227" s="3">
+        <v>980000</v>
+      </c>
+      <c r="H1227" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="I1227" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1227" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1227" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1227" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="M1227" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1228" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1228" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1228" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1228" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E1228" s="2">
+        <v>43</v>
+      </c>
+      <c r="F1228" s="3">
+        <v>2460000</v>
+      </c>
+      <c r="G1228" s="3">
+        <v>2450000</v>
+      </c>
+      <c r="H1228" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="I1228" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1228" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1228" s="2">
+        <v>1</v>
+      </c>
+      <c r="L1228" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="M1228" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1229" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1229" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1229" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1229" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E1229" s="2">
+        <v>42</v>
+      </c>
+      <c r="F1229" s="3">
+        <v>5300000</v>
+      </c>
+      <c r="G1229" s="3">
+        <v>5240000</v>
+      </c>
+      <c r="H1229" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="I1229" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1229" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1229" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1229" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="M1229" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1230" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1230" s="2" t="s">
+        <v>220</v>
+      </c>
+      <c r="C1230" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1230" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="E1230" s="2">
+        <v>43</v>
+      </c>
+      <c r="F1230" s="3">
+        <v>3930000</v>
+      </c>
+      <c r="G1230" s="3">
+        <v>3940000</v>
+      </c>
+      <c r="H1230" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="I1230" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1230" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="K1230" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1230" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="M1230" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1231" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1231" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="C1231" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1231" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="E1231" s="2">
+        <v>60</v>
+      </c>
+      <c r="F1231" s="3">
+        <v>1290000</v>
+      </c>
+      <c r="G1231" s="3">
+        <v>1280000</v>
+      </c>
+      <c r="H1231" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="I1231" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1231" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1231" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1231" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="M1231" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1232" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1232" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C1232" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1232" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="E1232" s="2">
+        <v>124</v>
+      </c>
+      <c r="F1232" s="3">
+        <v>3360000</v>
+      </c>
+      <c r="G1232" s="3">
+        <v>3290000</v>
+      </c>
+      <c r="H1232" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="I1232" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1232" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1232" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1232" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="M1232" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1233" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1233" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="C1233" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1233" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="E1233" s="2">
+        <v>178</v>
+      </c>
+      <c r="F1233" s="3">
+        <v>13520000</v>
+      </c>
+      <c r="G1233" s="3">
+        <v>13650000</v>
+      </c>
+      <c r="H1233" s="2" t="s">
+        <v>236</v>
+      </c>
+      <c r="I1233" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1233" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1233" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1233" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="M1233" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1234" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1234" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1234" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1234" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E1234" s="2">
+        <v>112</v>
+      </c>
+      <c r="F1234" s="3">
+        <v>4470000</v>
+      </c>
+      <c r="G1234" s="3">
+        <v>4440000</v>
+      </c>
+      <c r="H1234" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="I1234" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1234" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1234" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1234" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="M1234" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1235" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1235" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="C1235" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1235" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="E1235" s="2">
+        <v>108</v>
+      </c>
+      <c r="F1235" s="3">
+        <v>3880000</v>
+      </c>
+      <c r="G1235" s="3">
+        <v>3830000</v>
+      </c>
+      <c r="H1235" s="2" t="s">
+        <v>264</v>
+      </c>
+      <c r="I1235" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1235" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1235" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1235" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="M1235" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1236" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1236" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="C1236" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1236" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="E1236" s="2">
+        <v>183</v>
+      </c>
+      <c r="F1236" s="3">
+        <v>10010000</v>
+      </c>
+      <c r="G1236" s="3">
+        <v>9990000</v>
+      </c>
+      <c r="H1236" s="2" t="s">
+        <v>236</v>
+      </c>
+      <c r="I1236" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1236" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="K1236" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1236" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="M1236" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1237" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1237" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="C1237" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1237" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E1237" s="2">
+        <v>167</v>
+      </c>
+      <c r="F1237" s="3">
+        <v>9300000</v>
+      </c>
+      <c r="G1237" s="3">
+        <v>9150000</v>
+      </c>
+      <c r="H1237" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="I1237" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1237" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1237" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1237" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="M1237" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1238" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1238" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C1238" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1238" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="E1238" s="2">
+        <v>127</v>
+      </c>
+      <c r="F1238" s="3">
+        <v>3070000</v>
+      </c>
+      <c r="G1238" s="3">
+        <v>2980000</v>
+      </c>
+      <c r="H1238" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="I1238" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1238" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1238" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1238" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="M1238" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1239" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1239" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="C1239" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1239" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E1239" s="2">
+        <v>69</v>
+      </c>
+      <c r="F1239" s="3">
+        <v>1770000</v>
+      </c>
+      <c r="G1239" s="3">
+        <v>1780000</v>
+      </c>
+      <c r="H1239" s="2" t="s">
+        <v>241</v>
+      </c>
+      <c r="I1239" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1239" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1239" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1239" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="M1239" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1240" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1240" s="2" t="s">
+        <v>295</v>
+      </c>
+      <c r="C1240" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1240" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="E1240" s="2">
+        <v>100</v>
+      </c>
+      <c r="F1240" s="3">
+        <v>2580000</v>
+      </c>
+      <c r="G1240" s="3">
+        <v>2560000</v>
+      </c>
+      <c r="H1240" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="I1240" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1240" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1240" s="2">
+        <v>2</v>
+      </c>
+      <c r="L1240" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1240" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1241" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1241" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C1241" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1241" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="E1241" s="2">
+        <v>72</v>
+      </c>
+      <c r="F1241" s="3">
+        <v>1840000</v>
+      </c>
+      <c r="G1241" s="3">
+        <v>1840000</v>
+      </c>
+      <c r="H1241" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="I1241" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1241" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1241" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1241" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="M1241" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1242" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1242" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="C1242" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1242" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="E1242" s="2">
+        <v>0</v>
+      </c>
+      <c r="F1242" s="3">
+        <v>2510000</v>
+      </c>
+      <c r="G1242" s="3">
+        <v>2570000</v>
+      </c>
+      <c r="H1242" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="I1242" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1242" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1242" s="2">
+        <v>1</v>
+      </c>
+      <c r="L1242" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="M1242" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1243" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1243" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="C1243" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1243" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="E1243" s="2">
+        <v>0</v>
+      </c>
+      <c r="F1243" s="3">
+        <v>2000000</v>
+      </c>
+      <c r="G1243" s="3">
+        <v>2000000</v>
+      </c>
+      <c r="H1243" s="2" t="s">
+        <v>244</v>
+      </c>
+      <c r="I1243" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1243" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="K1243" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1243" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="M1243" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1244" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1244" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C1244" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1244" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="E1244" s="2">
+        <v>110</v>
+      </c>
+      <c r="F1244" s="3">
+        <v>3390000</v>
+      </c>
+      <c r="G1244" s="3">
+        <v>3340000</v>
+      </c>
+      <c r="H1244" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="I1244" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1244" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1244" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1244" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="M1244" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1245" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1245" s="2" t="s">
+        <v>284</v>
+      </c>
+      <c r="C1245" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1245" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1245" s="2">
+        <v>0</v>
+      </c>
+      <c r="F1245" s="3">
+        <v>3510000</v>
+      </c>
+      <c r="G1245" s="3">
+        <v>3510000</v>
+      </c>
+      <c r="H1245" s="2" t="s">
+        <v>285</v>
+      </c>
+      <c r="I1245" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1245" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1245" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1245" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="M1245" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1246" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1246" s="2" t="s">
+        <v>275</v>
+      </c>
+      <c r="C1246" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1246" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="E1246" s="2">
+        <v>59</v>
+      </c>
+      <c r="F1246" s="3">
+        <v>850000</v>
+      </c>
+      <c r="G1246" s="3">
+        <v>850000</v>
+      </c>
+      <c r="H1246" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="I1246" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1246" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1246" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1246" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="M1246" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1247" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1247" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C1247" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1247" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1247" s="2">
+        <v>0</v>
+      </c>
+      <c r="F1247" s="3">
+        <v>3030000</v>
+      </c>
+      <c r="G1247" s="3">
+        <v>2980000</v>
+      </c>
+      <c r="H1247" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="I1247" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1247" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1247" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1247" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="M1247" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1248" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1248" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="C1248" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1248" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="E1248" s="2">
+        <v>95</v>
+      </c>
+      <c r="F1248" s="3">
+        <v>3490000</v>
+      </c>
+      <c r="G1248" s="3">
+        <v>3470000</v>
+      </c>
+      <c r="H1248" s="2" t="s">
+        <v>285</v>
+      </c>
+      <c r="I1248" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1248" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1248" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1248" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="M1248" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1249" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1249" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="C1249" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1249" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="E1249" s="2">
+        <v>71</v>
+      </c>
+      <c r="F1249" s="3">
+        <v>1540000</v>
+      </c>
+      <c r="G1249" s="3">
+        <v>1550000</v>
+      </c>
+      <c r="H1249" s="2" t="s">
+        <v>238</v>
+      </c>
+      <c r="I1249" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1249" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1249" s="2">
+        <v>1</v>
+      </c>
+      <c r="L1249" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="M1249" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1250" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1250" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C1250" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1250" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="E1250" s="2">
+        <v>127</v>
+      </c>
+      <c r="F1250" s="3">
+        <v>5460000</v>
+      </c>
+      <c r="G1250" s="3">
+        <v>5360000</v>
+      </c>
+      <c r="H1250" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="I1250" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1250" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1250" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1250" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="M1250" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1251" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1251" s="2" t="s">
+        <v>303</v>
+      </c>
+      <c r="C1251" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1251" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="E1251" s="2">
+        <v>55</v>
+      </c>
+      <c r="F1251" s="3">
+        <v>630000</v>
+      </c>
+      <c r="G1251" s="3">
+        <v>640000</v>
+      </c>
+      <c r="H1251" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="I1251" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1251" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1251" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1251" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1251" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1252" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1252" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C1252" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1252" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="E1252" s="2">
+        <v>8</v>
+      </c>
+      <c r="F1252" s="3">
+        <v>220000</v>
+      </c>
+      <c r="G1252" s="3">
+        <v>220000</v>
+      </c>
+      <c r="H1252" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="I1252" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1252" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1252" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1252" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="M1252" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1253" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1253" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C1253" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1253" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="E1253" s="2">
+        <v>72</v>
+      </c>
+      <c r="F1253" s="3">
+        <v>2900000</v>
+      </c>
+      <c r="G1253" s="3">
+        <v>2800000</v>
+      </c>
+      <c r="H1253" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="I1253" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1253" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1253" s="2">
+        <v>1</v>
+      </c>
+      <c r="L1253" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="M1253" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1254" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1254" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="C1254" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1254" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="E1254" s="2">
+        <v>36</v>
+      </c>
+      <c r="F1254" s="3">
+        <v>3190000</v>
+      </c>
+      <c r="G1254" s="3">
+        <v>3230000</v>
+      </c>
+      <c r="H1254" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="I1254" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1254" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="K1254" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1254" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="M1254" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1255" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1255" s="2" t="s">
+        <v>286</v>
+      </c>
+      <c r="C1255" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1255" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="E1255" s="2">
+        <v>184</v>
+      </c>
+      <c r="F1255" s="3">
+        <v>15550000</v>
+      </c>
+      <c r="G1255" s="3">
+        <v>15560000</v>
+      </c>
+      <c r="H1255" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="I1255" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1255" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1255" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1255" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="M1255" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1256" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1256" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="C1256" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1256" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="E1256" s="2">
+        <v>87</v>
+      </c>
+      <c r="F1256" s="3">
+        <v>2650000</v>
+      </c>
+      <c r="G1256" s="3">
+        <v>2650000</v>
+      </c>
+      <c r="H1256" s="2" t="s">
+        <v>238</v>
+      </c>
+      <c r="I1256" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1256" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1256" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1256" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="M1256" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1257" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1257" s="2" t="s">
+        <v>296</v>
+      </c>
+      <c r="C1257" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1257" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="E1257" s="2">
+        <v>95</v>
+      </c>
+      <c r="F1257" s="3">
+        <v>7190000</v>
+      </c>
+      <c r="G1257" s="3">
+        <v>7200000</v>
+      </c>
+      <c r="H1257" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="I1257" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="J1257" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="K1257" s="2">
+        <v>2</v>
+      </c>
+      <c r="L1257" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1257" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1258" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1258" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="C1258" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1258" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="E1258" s="2">
+        <v>123</v>
+      </c>
+      <c r="F1258" s="3">
+        <v>3840000</v>
+      </c>
+      <c r="G1258" s="3">
+        <v>3880000</v>
+      </c>
+      <c r="H1258" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="I1258" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1258" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1258" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1258" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="M1258" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1259" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1259" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="C1259" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1259" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="E1259" s="2">
+        <v>89</v>
+      </c>
+      <c r="F1259" s="3">
+        <v>1650000</v>
+      </c>
+      <c r="G1259" s="3">
+        <v>1660000</v>
+      </c>
+      <c r="H1259" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="I1259" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1259" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1259" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1259" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="M1259" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1260" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1260" s="2" t="s">
+        <v>288</v>
+      </c>
+      <c r="C1260" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1260" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="E1260" s="2">
+        <v>0</v>
+      </c>
+      <c r="F1260" s="3">
+        <v>200000</v>
+      </c>
+      <c r="G1260" s="3">
+        <v>200000</v>
+      </c>
+      <c r="H1260" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="I1260" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1260" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="K1260" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1260" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1260" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1261" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1261" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="C1261" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1261" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E1261" s="2">
+        <v>100</v>
+      </c>
+      <c r="F1261" s="3">
+        <v>4790000</v>
+      </c>
+      <c r="G1261" s="3">
+        <v>4850000</v>
+      </c>
+      <c r="H1261" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="I1261" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1261" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1261" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1261" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="M1261" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1262" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1262" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="C1262" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1262" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1262" s="2">
+        <v>199</v>
+      </c>
+      <c r="F1262" s="3">
+        <v>18860000</v>
+      </c>
+      <c r="G1262" s="3">
+        <v>19090000</v>
+      </c>
+      <c r="H1262" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="I1262" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1262" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1262" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1262" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="M1262" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1263" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1263" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="C1263" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1263" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="E1263" s="2">
+        <v>179</v>
+      </c>
+      <c r="F1263" s="3">
+        <v>11600000</v>
+      </c>
+      <c r="G1263" s="3">
+        <v>11650000</v>
+      </c>
+      <c r="H1263" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="I1263" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1263" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1263" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1263" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="M1263" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1264" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1264" s="2" t="s">
+        <v>297</v>
+      </c>
+      <c r="C1264" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1264" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="E1264" s="2">
+        <v>46</v>
+      </c>
+      <c r="F1264" s="3">
+        <v>1330000</v>
+      </c>
+      <c r="G1264" s="3">
+        <v>1320000</v>
+      </c>
+      <c r="H1264" s="2" t="s">
+        <v>271</v>
+      </c>
+      <c r="I1264" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1264" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1264" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1264" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1264" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1265" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1265" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="C1265" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1265" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E1265" s="2">
+        <v>185</v>
+      </c>
+      <c r="F1265" s="3">
+        <v>12120000</v>
+      </c>
+      <c r="G1265" s="3">
+        <v>12080000</v>
+      </c>
+      <c r="H1265" s="2" t="s">
+        <v>255</v>
+      </c>
+      <c r="I1265" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1265" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1265" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1265" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="M1265" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1266" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1266" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="C1266" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1266" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1266" s="2">
+        <v>0</v>
+      </c>
+      <c r="F1266" s="3">
+        <v>4130000</v>
+      </c>
+      <c r="G1266" s="3">
+        <v>4180000</v>
+      </c>
+      <c r="H1266" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="I1266" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1266" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1266" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1266" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="M1266" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1267" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1267" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="C1267" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1267" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E1267" s="2">
+        <v>51</v>
+      </c>
+      <c r="F1267" s="3">
+        <v>2540000</v>
+      </c>
+      <c r="G1267" s="3">
+        <v>2570000</v>
+      </c>
+      <c r="H1267" s="2" t="s">
+        <v>246</v>
+      </c>
+      <c r="I1267" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1267" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1267" s="2">
+        <v>1</v>
+      </c>
+      <c r="L1267" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="M1267" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1268" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1268" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="C1268" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1268" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E1268" s="2">
+        <v>119</v>
+      </c>
+      <c r="F1268" s="3">
+        <v>5810000</v>
+      </c>
+      <c r="G1268" s="3">
+        <v>5790000</v>
+      </c>
+      <c r="H1268" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="I1268" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1268" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1268" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1268" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="M1268" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1269" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1269" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="C1269" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1269" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E1269" s="2">
+        <v>127</v>
+      </c>
+      <c r="F1269" s="3">
+        <v>6520000</v>
+      </c>
+      <c r="G1269" s="3">
+        <v>6400000</v>
+      </c>
+      <c r="H1269" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="I1269" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1269" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1269" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1269" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="M1269" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1270" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1270" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="C1270" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1270" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E1270" s="2">
+        <v>69</v>
+      </c>
+      <c r="F1270" s="3">
+        <v>4890000</v>
+      </c>
+      <c r="G1270" s="3">
+        <v>4880000</v>
+      </c>
+      <c r="H1270" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="I1270" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1270" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1270" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1270" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="M1270" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1271" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1271" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="C1271" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1271" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1271" s="2">
+        <v>68</v>
+      </c>
+      <c r="F1271" s="3">
+        <v>4330000</v>
+      </c>
+      <c r="G1271" s="3">
+        <v>4360000</v>
+      </c>
+      <c r="H1271" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="I1271" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1271" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="K1271" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1271" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="M1271" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1272" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1272" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="C1272" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1272" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="E1272" s="2">
+        <v>81</v>
+      </c>
+      <c r="F1272" s="3">
+        <v>1600000</v>
+      </c>
+      <c r="G1272" s="3">
+        <v>1610000</v>
+      </c>
+      <c r="H1272" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="I1272" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1272" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1272" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1272" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="M1272" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1273" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1273" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="C1273" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1273" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="E1273" s="2">
+        <v>123</v>
+      </c>
+      <c r="F1273" s="3">
+        <v>5280000</v>
+      </c>
+      <c r="G1273" s="3">
+        <v>5220000</v>
+      </c>
+      <c r="H1273" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="I1273" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1273" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1273" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1273" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="M1273" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1274" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1274" s="2" t="s">
+        <v>289</v>
+      </c>
+      <c r="C1274" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1274" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="E1274" s="2">
+        <v>128</v>
+      </c>
+      <c r="F1274" s="3">
+        <v>4760000</v>
+      </c>
+      <c r="G1274" s="3">
+        <v>4780000</v>
+      </c>
+      <c r="H1274" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="I1274" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1274" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1274" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1274" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="M1274" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1275" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1275" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="C1275" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1275" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="E1275" s="2">
+        <v>109</v>
+      </c>
+      <c r="F1275" s="3">
+        <v>3700000</v>
+      </c>
+      <c r="G1275" s="3">
+        <v>3650000</v>
+      </c>
+      <c r="H1275" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="I1275" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1275" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1275" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1275" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="M1275" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1276" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1276" s="2" t="s">
+        <v>290</v>
+      </c>
+      <c r="C1276" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1276" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1276" s="2">
+        <v>0</v>
+      </c>
+      <c r="F1276" s="3">
+        <v>170000</v>
+      </c>
+      <c r="G1276" s="3">
+        <v>170000</v>
+      </c>
+      <c r="H1276" s="2" t="s">
+        <v>291</v>
+      </c>
+      <c r="I1276" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1276" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="K1276" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1276" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1276" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1277" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1277" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="C1277" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1277" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E1277" s="2">
+        <v>36</v>
+      </c>
+      <c r="F1277" s="3">
+        <v>450000</v>
+      </c>
+      <c r="G1277" s="3">
+        <v>450000</v>
+      </c>
+      <c r="H1277" s="2" t="s">
+        <v>247</v>
+      </c>
+      <c r="I1277" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1277" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1277" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1277" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="M1277" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1278" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1278" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="C1278" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1278" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E1278" s="2">
+        <v>16</v>
+      </c>
+      <c r="F1278" s="3">
+        <v>430000</v>
+      </c>
+      <c r="G1278" s="3">
+        <v>430000</v>
+      </c>
+      <c r="H1278" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="I1278" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1278" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1278" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1278" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="M1278" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1279" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1279" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="C1279" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1279" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E1279" s="2">
+        <v>0</v>
+      </c>
+      <c r="F1279" s="3">
+        <v>2110000</v>
+      </c>
+      <c r="G1279" s="3">
+        <v>2110000</v>
+      </c>
+      <c r="H1279" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="I1279" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1279" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="K1279" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1279" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="M1279" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1280" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1280" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="C1280" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1280" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="E1280" s="2">
+        <v>12</v>
+      </c>
+      <c r="F1280" s="3">
+        <v>790000</v>
+      </c>
+      <c r="G1280" s="3">
+        <v>780000</v>
+      </c>
+      <c r="H1280" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="I1280" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1280" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1280" s="2">
+        <v>1</v>
+      </c>
+      <c r="L1280" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="M1280" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1281" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1281" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="C1281" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1281" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E1281" s="2">
+        <v>0</v>
+      </c>
+      <c r="F1281" s="3">
+        <v>9990000</v>
+      </c>
+      <c r="G1281" s="3">
+        <v>10060000</v>
+      </c>
+      <c r="H1281" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="I1281" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1281" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="K1281" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1281" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="M1281" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1282" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1282" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="C1282" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1282" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E1282" s="2">
+        <v>118</v>
+      </c>
+      <c r="F1282" s="3">
+        <v>6510000</v>
+      </c>
+      <c r="G1282" s="3">
+        <v>6370000</v>
+      </c>
+      <c r="H1282" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="I1282" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1282" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1282" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1282" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="M1282" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1283" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1283" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="C1283" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1283" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E1283" s="2">
+        <v>30</v>
+      </c>
+      <c r="F1283" s="3">
+        <v>2610000</v>
+      </c>
+      <c r="G1283" s="3">
+        <v>2740000</v>
+      </c>
+      <c r="H1283" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="I1283" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1283" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1283" s="2">
+        <v>1</v>
+      </c>
+      <c r="L1283" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="M1283" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1284" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1284" s="2" t="s">
+        <v>298</v>
+      </c>
+      <c r="C1284" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1284" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="E1284" s="2">
+        <v>0</v>
+      </c>
+      <c r="F1284" s="3">
+        <v>160000</v>
+      </c>
+      <c r="G1284" s="3">
+        <v>160000</v>
+      </c>
+      <c r="H1284" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="I1284" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1284" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="K1284" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1284" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1284" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1285" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1285" s="2" t="s">
+        <v>304</v>
+      </c>
+      <c r="C1285" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1285" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="E1285" s="2">
+        <v>26</v>
+      </c>
+      <c r="F1285" s="3">
+        <v>320000</v>
+      </c>
+      <c r="G1285" s="3">
+        <v>320000</v>
+      </c>
+      <c r="H1285" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="I1285" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1285" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1285" s="2">
+        <v>5</v>
+      </c>
+      <c r="L1285" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1285" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1286" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1286" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="C1286" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1286" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E1286" s="2">
+        <v>54</v>
+      </c>
+      <c r="F1286" s="3">
+        <v>2350000</v>
+      </c>
+      <c r="G1286" s="3">
+        <v>2330000</v>
+      </c>
+      <c r="H1286" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="I1286" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1286" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1286" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1286" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="M1286" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1287" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1287" s="2" t="s">
+        <v>305</v>
+      </c>
+      <c r="C1287" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1287" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1287" s="2">
+        <v>131</v>
+      </c>
+      <c r="F1287" s="3">
+        <v>5090000</v>
+      </c>
+      <c r="G1287" s="3">
+        <v>5040000</v>
+      </c>
+      <c r="H1287" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="I1287" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1287" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1287" s="2">
+        <v>1</v>
+      </c>
+      <c r="L1287" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1287" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1288" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1288" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="C1288" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1288" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E1288" s="2">
+        <v>89</v>
+      </c>
+      <c r="F1288" s="3">
+        <v>8280000</v>
+      </c>
+      <c r="G1288" s="3">
+        <v>8280000</v>
+      </c>
+      <c r="H1288" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="I1288" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1288" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1288" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1288" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="M1288" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1289" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1289" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="C1289" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1289" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="E1289" s="2">
+        <v>130</v>
+      </c>
+      <c r="F1289" s="3">
+        <v>11240000</v>
+      </c>
+      <c r="G1289" s="3">
+        <v>11300000</v>
+      </c>
+      <c r="H1289" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="I1289" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1289" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="K1289" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1289" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="M1289" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1290" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1290" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="C1290" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1290" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1290" s="2">
+        <v>0</v>
+      </c>
+      <c r="F1290" s="3">
+        <v>2020000</v>
+      </c>
+      <c r="G1290" s="3">
+        <v>1990000</v>
+      </c>
+      <c r="H1290" s="2" t="s">
+        <v>241</v>
+      </c>
+      <c r="I1290" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1290" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1290" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1290" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="M1290" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1291" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1291" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="C1291" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1291" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="E1291" s="2">
+        <v>41</v>
+      </c>
+      <c r="F1291" s="3">
+        <v>1160000</v>
+      </c>
+      <c r="G1291" s="3">
+        <v>1130000</v>
+      </c>
+      <c r="H1291" s="2" t="s">
+        <v>285</v>
+      </c>
+      <c r="I1291" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1291" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1291" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1291" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="M1291" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1292" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1292" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="C1292" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1292" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1292" s="2">
+        <v>91</v>
+      </c>
+      <c r="F1292" s="3">
+        <v>8180000</v>
+      </c>
+      <c r="G1292" s="3">
+        <v>8120000</v>
+      </c>
+      <c r="H1292" s="2" t="s">
+        <v>264</v>
+      </c>
+      <c r="I1292" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1292" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1292" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1292" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="M1292" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1293" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1293" s="2" t="s">
+        <v>292</v>
+      </c>
+      <c r="C1293" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1293" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="E1293" s="2">
+        <v>30</v>
+      </c>
+      <c r="F1293" s="3">
+        <v>830000</v>
+      </c>
+      <c r="G1293" s="3">
+        <v>830000</v>
+      </c>
+      <c r="H1293" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="I1293" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1293" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1293" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1293" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="M1293" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1294" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1294" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="C1294" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1294" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="E1294" s="2">
+        <v>1</v>
+      </c>
+      <c r="F1294" s="3">
+        <v>280000</v>
+      </c>
+      <c r="G1294" s="3">
+        <v>280000</v>
+      </c>
+      <c r="H1294" s="2" t="s">
+        <v>244</v>
+      </c>
+      <c r="I1294" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1294" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="K1294" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1294" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="M1294" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1295" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1295" s="2" t="s">
+        <v>299</v>
+      </c>
+      <c r="C1295" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1295" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E1295" s="2">
+        <v>0</v>
+      </c>
+      <c r="F1295" s="3">
+        <v>160000</v>
+      </c>
+      <c r="G1295" s="3">
+        <v>160000</v>
+      </c>
+      <c r="H1295" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="I1295" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1295" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="K1295" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1295" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1295" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1296" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1296" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="C1296" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1296" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="E1296" s="2">
+        <v>108</v>
+      </c>
+      <c r="F1296" s="3">
+        <v>3270000</v>
+      </c>
+      <c r="G1296" s="3">
+        <v>3210000</v>
+      </c>
+      <c r="H1296" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="I1296" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1296" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1296" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1296" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="M1296" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1297" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1297" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="C1297" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1297" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="E1297" s="2">
+        <v>112</v>
+      </c>
+      <c r="F1297" s="3">
+        <v>3890000</v>
+      </c>
+      <c r="G1297" s="3">
+        <v>3830000</v>
+      </c>
+      <c r="H1297" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="I1297" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="J1297" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1297" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1297" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="M1297" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1298" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1298" s="2" t="s">
+        <v>278</v>
+      </c>
+      <c r="C1298" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1298" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E1298" s="2">
+        <v>136</v>
+      </c>
+      <c r="F1298" s="3">
+        <v>7260000</v>
+      </c>
+      <c r="G1298" s="3">
+        <v>7260000</v>
+      </c>
+      <c r="H1298" s="2" t="s">
+        <v>279</v>
+      </c>
+      <c r="I1298" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1298" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1298" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1298" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="M1298" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1299" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1299" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="C1299" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1299" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="E1299" s="2">
+        <v>90</v>
+      </c>
+      <c r="F1299" s="3">
+        <v>3570000</v>
+      </c>
+      <c r="G1299" s="3">
+        <v>3550000</v>
+      </c>
+      <c r="H1299" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="I1299" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1299" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1299" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1299" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="M1299" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1300" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1300" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="C1300" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1300" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="E1300" s="2">
+        <v>15</v>
+      </c>
+      <c r="F1300" s="3">
+        <v>360000</v>
+      </c>
+      <c r="G1300" s="3">
+        <v>360000</v>
+      </c>
+      <c r="H1300" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="I1300" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1300" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1300" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1300" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="M1300" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1301" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1301" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="C1301" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1301" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="E1301" s="2">
+        <v>58</v>
+      </c>
+      <c r="F1301" s="3">
+        <v>1150000</v>
+      </c>
+      <c r="G1301" s="3">
+        <v>1150000</v>
+      </c>
+      <c r="H1301" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="I1301" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1301" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1301" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1301" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="M1301" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1302" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1302" s="2" t="s">
+        <v>293</v>
+      </c>
+      <c r="C1302" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1302" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="E1302" s="2">
+        <v>48</v>
+      </c>
+      <c r="F1302" s="3">
+        <v>1500000</v>
+      </c>
+      <c r="G1302" s="3">
+        <v>1480000</v>
+      </c>
+      <c r="H1302" s="2" t="s">
+        <v>246</v>
+      </c>
+      <c r="I1302" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1302" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1302" s="2">
+        <v>1</v>
+      </c>
+      <c r="L1302" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="M1302" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1303" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1303" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="C1303" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1303" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E1303" s="2">
+        <v>77</v>
+      </c>
+      <c r="F1303" s="3">
+        <v>4420000</v>
+      </c>
+      <c r="G1303" s="3">
+        <v>4440000</v>
+      </c>
+      <c r="H1303" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="I1303" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1303" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1303" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1303" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="M1303" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1304" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1304" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="C1304" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1304" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="E1304" s="2">
+        <v>4</v>
+      </c>
+      <c r="F1304" s="3">
+        <v>370000</v>
+      </c>
+      <c r="G1304" s="3">
+        <v>370000</v>
+      </c>
+      <c r="H1304" s="2" t="s">
+        <v>244</v>
+      </c>
+      <c r="I1304" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1304" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="K1304" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1304" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="M1304" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1305" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1305" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="C1305" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1305" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E1305" s="2">
+        <v>4</v>
+      </c>
+      <c r="F1305" s="3">
+        <v>390000</v>
+      </c>
+      <c r="G1305" s="3">
+        <v>390000</v>
+      </c>
+      <c r="H1305" s="2" t="s">
+        <v>268</v>
+      </c>
+      <c r="I1305" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1305" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1305" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1305" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="M1305" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1306" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1306" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="C1306" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1306" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E1306" s="2">
+        <v>156</v>
+      </c>
+      <c r="F1306" s="3">
+        <v>6890000</v>
+      </c>
+      <c r="G1306" s="3">
+        <v>6830000</v>
+      </c>
+      <c r="H1306" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="I1306" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1306" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1306" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1306" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="M1306" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1307" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1307" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="C1307" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1307" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="E1307" s="2">
+        <v>29</v>
+      </c>
+      <c r="F1307" s="3">
+        <v>760000</v>
+      </c>
+      <c r="G1307" s="3">
+        <v>750000</v>
+      </c>
+      <c r="H1307" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="I1307" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1307" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1307" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1307" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="M1307" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1308" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1308" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="C1308" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1308" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E1308" s="2">
+        <v>102</v>
+      </c>
+      <c r="F1308" s="3">
+        <v>3010000</v>
+      </c>
+      <c r="G1308" s="3">
+        <v>2960000</v>
+      </c>
+      <c r="H1308" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="I1308" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1308" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1308" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1308" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="M1308" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1309" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1309" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="C1309" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1309" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="E1309" s="2">
+        <v>19</v>
+      </c>
+      <c r="F1309" s="3">
+        <v>900000</v>
+      </c>
+      <c r="G1309" s="3">
+        <v>890000</v>
+      </c>
+      <c r="H1309" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="I1309" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1309" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1309" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1309" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="M1309" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1310" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1310" s="2" t="s">
+        <v>306</v>
+      </c>
+      <c r="C1310" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1310" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="E1310" s="2">
+        <v>0</v>
+      </c>
+      <c r="F1310" s="3">
+        <v>190000</v>
+      </c>
+      <c r="G1310" s="3">
+        <v>190000</v>
+      </c>
+      <c r="H1310" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="I1310" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1310" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="K1310" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1310" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1310" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1311" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1311" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="C1311" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1311" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E1311" s="2">
+        <v>11</v>
+      </c>
+      <c r="F1311" s="3">
+        <v>2890000</v>
+      </c>
+      <c r="G1311" s="3">
+        <v>2850000</v>
+      </c>
+      <c r="H1311" s="2" t="s">
+        <v>265</v>
+      </c>
+      <c r="I1311" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1311" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="K1311" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1311" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="M1311" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1312" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1312" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="C1312" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1312" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="E1312" s="2">
+        <v>17</v>
+      </c>
+      <c r="F1312" s="3">
+        <v>1280000</v>
+      </c>
+      <c r="G1312" s="3">
+        <v>1260000</v>
+      </c>
+      <c r="H1312" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="I1312" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1312" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1312" s="2">
+        <v>1</v>
+      </c>
+      <c r="L1312" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="M1312" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1313" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1313" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="C1313" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1313" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="E1313" s="2">
+        <v>0</v>
+      </c>
+      <c r="F1313" s="3">
+        <v>160000</v>
+      </c>
+      <c r="G1313" s="3">
+        <v>160000</v>
+      </c>
+      <c r="H1313" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="I1313" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1313" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="K1313" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1313" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1313" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1314" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1314" s="2" t="s">
+        <v>307</v>
+      </c>
+      <c r="C1314" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1314" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1314" s="2">
+        <v>0</v>
+      </c>
+      <c r="F1314" s="3">
+        <v>160000</v>
+      </c>
+      <c r="G1314" s="3">
+        <v>160000</v>
+      </c>
+      <c r="H1314" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="I1314" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1314" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="K1314" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1314" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1314" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1315" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1315" s="2" t="s">
+        <v>300</v>
+      </c>
+      <c r="C1315" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1315" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1315" s="2">
+        <v>0</v>
+      </c>
+      <c r="F1315" s="3">
+        <v>410000</v>
+      </c>
+      <c r="G1315" s="3">
+        <v>410000</v>
+      </c>
+      <c r="H1315" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="I1315" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1315" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="K1315" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1315" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M1315" s="7" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="1316" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1316" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="C1316" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1316" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="E1316" s="2">
+        <v>0</v>
+      </c>
+      <c r="F1316" s="3">
+        <v>3380000</v>
+      </c>
+      <c r="G1316" s="3">
+        <v>3380000</v>
+      </c>
+      <c r="H1316" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="I1316" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1316" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="K1316" s="2">
+        <v>0</v>
+      </c>
+      <c r="L1316" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="M1316" s="7" t="s">
+        <v>308</v>
       </c>
     </row>
   </sheetData>

</xml_diff>